<commit_message>
Add Bangalore location lens: sort Tier 1 Bangalore-first, annotate fit
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Kq1GVuDP62P4fjx7tfK9jZ
</commit_message>
<xml_diff>
--- a/outreach/target-companies-tracker.xlsx
+++ b/outreach/target-companies-tracker.xlsx
@@ -53,7 +53,7 @@
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -63,6 +63,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DEEAF6"/>
       </patternFill>
     </fill>
     <fill>
@@ -97,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -110,6 +115,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -486,24 +494,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O26"/>
+  <dimension ref="A1:P26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="26" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="30" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="26" customWidth="1" min="15" max="15"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="30" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="26" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -524,60 +533,65 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Bangalore Fit</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Why It Made the List (Growth Signal)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Funding / Profitability</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Role Fit</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Comp Signal</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Reviews Check (G2 / Glassdoor / RepVue)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Risk Flags</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Who to Reach (Titles)</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Outreach Angle</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Next Step</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>My Notes</t>
         </is>
@@ -597,62 +611,67 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Bangalore office</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>Global — HR/IT/Fin platform</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>~53 open Bengaluru roles incl. Mid-Market AE and SDR Manager (Outbound); Bangalore hub sells outbound into North America SMB/MM</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>Late-stage, hypergrowth</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>SDR Manager + MM AE (both open)</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>SDR median base ~Rs14L; India avg total comp ~Rs59L (6figr)</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="J2" s="4" t="inlineStr">
         <is>
           <t>Check RepVue + Glassdoor sales filter; strong pay reports</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="K2" s="4" t="inlineStr">
         <is>
           <t>Intense pace; hybrid 3 days/office; Deel litigation noise</t>
         </is>
       </c>
-      <c r="K2" s="4" t="inlineStr">
+      <c r="L2" s="4" t="inlineStr">
         <is>
           <t>Head of Sales Dev India; India GTM site lead</t>
         </is>
       </c>
-      <c r="L2" s="4" t="inlineStr">
+      <c r="M2" s="4" t="inlineStr">
         <is>
           <t>Outbound playbook + team leadership story maps 1:1 to their outbound SMB motion</t>
         </is>
       </c>
-      <c r="M2" s="5" t="inlineStr">
+      <c r="N2" s="6" t="inlineStr">
         <is>
           <t>Contacted</t>
         </is>
       </c>
-      <c r="N2" s="5" t="inlineStr">
+      <c r="O2" s="6" t="inlineStr">
         <is>
           <t>Follow up 28-Jul if no reply</t>
         </is>
       </c>
-      <c r="O2" s="5" t="inlineStr">
+      <c r="P2" s="6" t="inlineStr">
         <is>
           <t>e.g. Emailed Head of Sales Dev 21-Jul via LinkedIn</t>
         </is>
@@ -672,58 +691,63 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Bangalore office</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>Global — Data/AI</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>Among fastest-growing software cos ever; AI tailwind; 3,000+ India job listings; India-market BDR hiring seen</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>Pre-IPO, massively funded</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>BDR lead / commercial AE</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>Top-of-market + pre-IPO equity</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="J3" s="4" t="inlineStr">
         <is>
           <t>Strong employer brand; verify India sales Glassdoor</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="K3" s="4" t="inlineStr">
         <is>
           <t>AE seats may be senior; India GTM younger than R&amp;D</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="L3" s="4" t="inlineStr">
         <is>
           <t>RVP India / India sales leadership</t>
         </is>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="M3" s="4" t="inlineStr">
         <is>
           <t>AI category momentum; ask about GTM build-out as India scales</t>
         </is>
       </c>
-      <c r="M3" s="5" t="inlineStr">
+      <c r="N3" s="6" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="N3" s="5" t="n"/>
-      <c r="O3" s="5" t="n"/>
+      <c r="O3" s="6" t="n"/>
+      <c r="P3" s="6" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -739,58 +763,63 @@
           <t>Bengaluru / Mumbai</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Bangalore office</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Global — Data cloud</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>SDR role open in Bengaluru (posted Jun 2026); public, growing, FCF positive</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>Public, profitable on FCF</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>SDR leadership path; commercial AE</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Enterprise AE OTEs high (India ent. AE median OTE ~Rs65L)</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>Solid RepVue historically</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>AE seats skew senior enterprise</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>SDR Manager India; Country Mgr</t>
         </is>
       </c>
-      <c r="L4" s="4" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>Enterprise motion experience + outbound rigor</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="N4" s="6" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="N4" s="5" t="n"/>
-      <c r="O4" s="5" t="n"/>
+      <c r="O4" s="6" t="n"/>
+      <c r="P4" s="6" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -806,58 +835,63 @@
           <t>Gurgaon / Bengaluru</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Bangalore office (verify sales seats; sales HQ Gurgaon)</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Global — Database</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>Established India-market sales org; best-known SDR-to-AE academy ladder in tech</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>Public, durable</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>SDR Mgr or AE via ladder</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>Competitive; RSUs</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>Historically strong RepVue</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>Growth moderated vs 2021 peaks</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>Regional Director India</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="M5" s="4" t="inlineStr">
         <is>
           <t>Their promotion ladder = your AE jump story</t>
         </is>
       </c>
-      <c r="M5" s="5" t="inlineStr">
+      <c r="N5" s="6" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="N5" s="5" t="n"/>
-      <c r="O5" s="5" t="n"/>
+      <c r="O5" s="6" t="n"/>
+      <c r="P5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -873,58 +907,63 @@
           <t>India (newer)</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Bangalore likely — verify</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>Global — Observability</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>RepVue quota attainment 83.7% (elite vs ~43% industry avg); profitable, ~25% growth</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>Public, profitable</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>Commercial AE</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>High; verify India bands</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="J6" s="4" t="inlineStr">
         <is>
           <t>RepVue elite</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="K6" s="4" t="inlineStr">
         <is>
           <t>India GTM footprint newer/smaller — verify openings</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="L6" s="4" t="inlineStr">
         <is>
           <t>APAC sales leadership</t>
         </is>
       </c>
-      <c r="L6" s="4" t="inlineStr">
+      <c r="M6" s="4" t="inlineStr">
         <is>
           <t>Attainment culture pitch: you want a quota that's real</t>
         </is>
       </c>
-      <c r="M6" s="5" t="inlineStr">
+      <c r="N6" s="6" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="N6" s="5" t="n"/>
-      <c r="O6" s="5" t="n"/>
+      <c r="O6" s="6" t="n"/>
+      <c r="P6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -940,58 +979,63 @@
           <t>Pune / Bengaluru</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Bangalore office</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>Global — ABM/Revenue AI</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>RepVue attainment 83.2%; large India presence; product sells to sales leaders (your persona)</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>Late-stage funded</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>BDR leadership; AE (verify)</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>Good; verify India bands</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="J7" s="4" t="inlineStr">
         <is>
           <t>RepVue elite</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr">
+      <c r="K7" s="4" t="inlineStr">
         <is>
           <t>India roles skew R&amp;D + BDR</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr">
+      <c r="L7" s="4" t="inlineStr">
         <is>
           <t>India site lead; Head of SDR</t>
         </is>
       </c>
-      <c r="L7" s="4" t="inlineStr">
+      <c r="M7" s="4" t="inlineStr">
         <is>
           <t>You ARE the ICP — sell sales-intelligence as a seller</t>
         </is>
       </c>
-      <c r="M7" s="5" t="inlineStr">
+      <c r="N7" s="6" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="N7" s="5" t="n"/>
-      <c r="O7" s="5" t="n"/>
+      <c r="O7" s="6" t="n"/>
+      <c r="P7" s="6" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -999,66 +1043,71 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Deel</t>
+          <t>Freshworks</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Remote (India)</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>Global — Payroll/EOR</t>
+          <t>Chennai / BLR / Hyd</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Bangalore office (HQ Chennai)</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>~$1B ARR, profitable; hires remote AEs/SDR leaders in India timezones for APAC/EMEA</t>
+          <t>India-HQ — CX/ITSM suite</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Profitable</t>
+          <t>Public; 16% YoY; EX business crossed $500M ARR; most mature sales career ladder in Indian SaaS</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Remote AE / SDR leader</t>
+          <t>Public, strong FCF</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Strong global-remote bands</t>
+          <t>SDR Mgr, AE, or Mgr track</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Check RepVue; fast-paced</t>
+          <t>Competitive at senior levels; liquid RSUs</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>Fully remote culture; Rippling feud</t>
+          <t>G2 strong across products; filter Glassdoor to sales</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>APAC sales leadership</t>
+          <t>Growth moderating; Nov-2024 restructure (~13%)</t>
         </is>
       </c>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>Remote + APAC coverage experience</t>
-        </is>
-      </c>
-      <c r="M8" s="5" t="inlineStr">
+          <t>Director Sales Dev; VP Sales (segment)</t>
+        </is>
+      </c>
+      <c r="M8" s="4" t="inlineStr">
+        <is>
+          <t>Ladder + brand; ask about MM AE or SDR leadership</t>
+        </is>
+      </c>
+      <c r="N8" s="6" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="N8" s="5" t="n"/>
-      <c r="O8" s="5" t="n"/>
+      <c r="O8" s="6" t="n"/>
+      <c r="P8" s="6" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1066,66 +1115,71 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Freshworks</t>
+          <t>Postman</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Chennai / BLR / Hyd</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>India-HQ — CX/ITSM suite</t>
+          <t>Bengaluru / SF</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Bangalore office</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Public; 16% YoY; EX business crossed $500M ARR; most mature sales career ladder in Indian SaaS</t>
+          <t>India-HQ — API platform</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Public, strong FCF</t>
+          <t>$5.6B val; AI Agent momentum (Agent Builder; Fern + liblab acquisitions); moving upmarket</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>SDR Mgr, AE, or Mgr track</t>
+          <t>Late-stage, efficient</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Competitive at senior levels; liquid RSUs</t>
+          <t>Enterprise AE; sales-dev leadership</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>G2 strong across products; filter Glassdoor to sales</t>
+          <t>Strong; equity story good</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>Growth moderating; Nov-2024 restructure (~13%)</t>
+          <t>G2 category leader; strong brand halo</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>Director Sales Dev; VP Sales (segment)</t>
+          <t>PLG DNA — sales org smaller</t>
         </is>
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>Ladder + brand; ask about MM AE or SDR leadership</t>
-        </is>
-      </c>
-      <c r="M9" s="5" t="inlineStr">
+          <t>CRO org; Head of Enterprise Sales</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="inlineStr">
+        <is>
+          <t>Enterprise motion is new-ish — early AE upside</t>
+        </is>
+      </c>
+      <c r="N9" s="6" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="N9" s="5" t="n"/>
-      <c r="O9" s="5" t="n"/>
+      <c r="O9" s="6" t="n"/>
+      <c r="P9" s="6" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -1133,66 +1187,71 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Postman</t>
+          <t>Sprinto</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Bengaluru / SF</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>India-HQ — API platform</t>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Bangalore HQ (remote-first)</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>$5.6B val; AI Agent momentum (Agent Builder; Fern + liblab acquisitions); moving upmarket</t>
+          <t>India-HQ — Compliance automation</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Late-stage, efficient</t>
+          <t>~$38M ARR compounding; outbound-heavy US SMB/MM motion — most BDR-manager-shaped org on list</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>Enterprise AE; sales-dev leadership</t>
+          <t>Series B, efficient</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>Strong; equity story good</t>
+          <t>SDR/BDR Manager (ideal); AE</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>G2 category leader; strong brand halo</t>
+          <t>Mid-to-good; verify OTE split</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>PLG DNA — sales org smaller</t>
+          <t>G2 strong vs Vanta/Drata</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>CRO org; Head of Enterprise Sales</t>
+          <t>Earlier stage; check attainment claims</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>Enterprise motion is new-ish — early AE upside</t>
-        </is>
-      </c>
-      <c r="M10" s="5" t="inlineStr">
+          <t>Founder; Head of Sales</t>
+        </is>
+      </c>
+      <c r="M10" s="4" t="inlineStr">
+        <is>
+          <t>Outbound org needs outbound leadership — direct fit</t>
+        </is>
+      </c>
+      <c r="N10" s="6" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="N10" s="5" t="n"/>
-      <c r="O10" s="5" t="n"/>
+      <c r="O10" s="6" t="n"/>
+      <c r="P10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1200,66 +1259,71 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>BrowserStack</t>
+          <t>MoEngage</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Mumbai / Dublin</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>India-HQ — Testing cloud</t>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Bangalore HQ</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Profitable; large India-based global inside-sales org; sells worldwide from India</t>
+          <t>India-HQ — Customer engagement</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Profitable</t>
+          <t>~$280M Series F (Dec 2025) — explicit GTM war chest; US/EU/SEA expansion</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>AE + SDR Manager roles recur</t>
+          <t>Series F, funded for GTM</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Competitive; sales org large enough for bands</t>
+          <t>AE (multiple geos); SDR Mgr</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>G2 strong in category</t>
+          <t>Competitive post-raise</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>Interview bar high; check sales Glassdoor</t>
+          <t>G2 solid; check Glassdoor sales</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>VP Inside Sales; Dir Sales Dev</t>
+          <t>Integration of big raise = org churn possible</t>
         </is>
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>Global-selling-from-India is their whole model</t>
-        </is>
-      </c>
-      <c r="M11" s="5" t="inlineStr">
+          <t>CRO; Regional VPs</t>
+        </is>
+      </c>
+      <c r="M11" s="4" t="inlineStr">
+        <is>
+          <t>Fresh capital earmarked for GTM = hiring wave</t>
+        </is>
+      </c>
+      <c r="N11" s="6" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="N11" s="5" t="n"/>
-      <c r="O11" s="5" t="n"/>
+      <c r="O11" s="6" t="n"/>
+      <c r="P11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1267,66 +1331,71 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Chargebee</t>
+          <t>Whatfix</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Chennai</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>India-HQ — Billing</t>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Bangalore HQ</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Gartner MQ Leader, Recurring Billing 2025; acquired Inai; global base sold from India</t>
+          <t>India-HQ — Digital adoption</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Late-stage</t>
+          <t>Pre-IPO (secondaries on EquityZen); AE 'GTM Labs' roles OPEN now; sells US enterprise</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>AE; SDR leadership</t>
+          <t>Pre-IPO</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Competitive</t>
+          <t>AE (open now)</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>MQ Leader; DO the Glassdoor sales-filter check</t>
+          <t>Competitive; pre-IPO equity</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>10% layoff late 2022</t>
+          <t>G2 DAP leader; check Glassdoor</t>
         </is>
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>VP Sales; Dir Sales Dev</t>
+          <t>IPO timing uncertain</t>
         </is>
       </c>
       <c r="L12" s="4" t="inlineStr">
         <is>
-          <t>MQ Leader momentum into enterprise billing deals</t>
-        </is>
-      </c>
-      <c r="M12" s="5" t="inlineStr">
+          <t>Talent team via open req; VP Sales</t>
+        </is>
+      </c>
+      <c r="M12" s="4" t="inlineStr">
+        <is>
+          <t>Live opening — apply + parallel warm intro</t>
+        </is>
+      </c>
+      <c r="N12" s="6" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="N12" s="5" t="n"/>
-      <c r="O12" s="5" t="n"/>
+      <c r="O12" s="6" t="n"/>
+      <c r="P12" s="6" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1334,66 +1403,71 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Rocketlane</t>
+          <t>DevRev</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Chennai</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>India-HQ — Onboarding/PSA</t>
+          <t>Bengaluru + US</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Bangalore office</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>$60M Series C (Mar 2026, Insight) after doubling revenue; ex-Freshworks founders, culture reputation</t>
+          <t>India-HQ — AI-native support/CRM</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Series C, fresh runway</t>
+          <t>Dheeraj Pandey (Nutanix founder); heavily funded; AI-native in hot category; GTM being built</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>AE (high impact, small team)</t>
+          <t>Well-funded, earlier GTM</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
-          <t>Mid; equity meaningful</t>
+          <t>Early AE (scope upside)</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>G2 momentum strong in PSA</t>
+          <t>Mid now, equity upside</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>Smaller org = less structure</t>
+          <t>Too early for deep review data</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
-          <t>Founder/CEO; VP Sales</t>
+          <t>Motion still forming — risk</t>
         </is>
       </c>
       <c r="L13" s="4" t="inlineStr">
         <is>
-          <t>Series-C GTM expansion = they need closers now</t>
-        </is>
-      </c>
-      <c r="M13" s="5" t="inlineStr">
+          <t>Founder office; Head of GTM</t>
+        </is>
+      </c>
+      <c r="M13" s="4" t="inlineStr">
+        <is>
+          <t>Early-AE bet on a proven founder</t>
+        </is>
+      </c>
+      <c r="N13" s="6" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="N13" s="5" t="n"/>
-      <c r="O13" s="5" t="n"/>
+      <c r="O13" s="6" t="n"/>
+      <c r="P13" s="6" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1401,66 +1475,71 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Sprinto</t>
+          <t>Everstage</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>India-HQ — Compliance automation</t>
+          <t>Chennai / BLR</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Bangalore presence (HQ Chennai)</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>~$38M ARR compounding; outbound-heavy US SMB/MM motion — most BDR-manager-shaped org on list</t>
+          <t>India-HQ — Sales commissions</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Series B, efficient</t>
+          <t>$44.7M raised; strong G2 momentum in incentive comp; ICP is RevOps + sales leaders</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>SDR/BDR Manager (ideal); AE</t>
+          <t>Series B</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>Mid-to-good; verify OTE split</t>
+          <t>AE — you are the ICP</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>G2 strong vs Vanta/Drata</t>
+          <t>Mid; verify</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>Earlier stage; check attainment claims</t>
+          <t>Strong G2 momentum</t>
         </is>
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
+          <t>Category has big incumbents (Xactly etc.)</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
           <t>Founder; Head of Sales</t>
         </is>
       </c>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t>Outbound org needs outbound leadership — direct fit</t>
-        </is>
-      </c>
-      <c r="M14" s="5" t="inlineStr">
+      <c r="M14" s="4" t="inlineStr">
+        <is>
+          <t>A rep who lived commission pain sells this best</t>
+        </is>
+      </c>
+      <c r="N14" s="6" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="N14" s="5" t="n"/>
-      <c r="O14" s="5" t="n"/>
+      <c r="O14" s="6" t="n"/>
+      <c r="P14" s="6" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1468,7 +1547,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>MoEngage</t>
+          <t>Amagi</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -1476,58 +1555,63 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>India-HQ — Customer engagement</t>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Bangalore HQ</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>~$280M Series F (Dec 2025) — explicit GTM war chest; US/EU/SEA expansion</t>
+          <t>India-HQ — Media cloud SaaS</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Series F, funded for GTM</t>
+          <t>Unicorn; turned profitable; IPO track; global media customers from India</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>AE (multiple geos); SDR Mgr</t>
+          <t>Profitable, IPO track</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>Competitive post-raise</t>
+          <t>AE (media vertical)</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>G2 solid; check Glassdoor sales</t>
+          <t>Competitive</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>Integration of big raise = org churn possible</t>
+          <t>Check G2/Glassdoor — vertical niche</t>
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>CRO; Regional VPs</t>
+          <t>Vertical = narrower ICP</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr">
         <is>
-          <t>Fresh capital earmarked for GTM = hiring wave</t>
-        </is>
-      </c>
-      <c r="M15" s="5" t="inlineStr">
+          <t>VP Sales</t>
+        </is>
+      </c>
+      <c r="M15" s="4" t="inlineStr">
+        <is>
+          <t>Vertical depth + profitability story</t>
+        </is>
+      </c>
+      <c r="N15" s="6" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="N15" s="5" t="n"/>
-      <c r="O15" s="5" t="n"/>
+      <c r="O15" s="6" t="n"/>
+      <c r="P15" s="6" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1535,66 +1619,71 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Darwinbox</t>
+          <t>Deel</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Hyderabad</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>India-HQ — Enterprise HR SaaS</t>
+          <t>Remote (India)</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Remote (India)</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>~$300M+ raised incl. 2025; enterprise machine across India/SEA/ME/US; real enterprise ACVs</t>
+          <t>Global — Payroll/EOR</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Late-stage</t>
+          <t>~$1B ARR, profitable; hires remote AEs/SDR leaders in India timezones for APAC/EMEA</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>Enterprise AE training ground</t>
+          <t>Profitable</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>Good enterprise OTEs</t>
+          <t>Remote AE / SDR leader</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>Check Glassdoor sales filter</t>
+          <t>Strong global-remote bands</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>Enterprise cycles are long; comp back-loaded</t>
+          <t>Check RepVue; fast-paced</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>VP Sales (region)</t>
+          <t>Fully remote culture; Rippling feud</t>
         </is>
       </c>
       <c r="L16" s="4" t="inlineStr">
         <is>
-          <t>Enterprise AE ambition + HR-tech domain interest</t>
-        </is>
-      </c>
-      <c r="M16" s="5" t="inlineStr">
+          <t>APAC sales leadership</t>
+        </is>
+      </c>
+      <c r="M16" s="4" t="inlineStr">
+        <is>
+          <t>Remote + APAC coverage experience</t>
+        </is>
+      </c>
+      <c r="N16" s="6" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="N16" s="5" t="n"/>
-      <c r="O16" s="5" t="n"/>
+      <c r="O16" s="6" t="n"/>
+      <c r="P16" s="6" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1602,66 +1691,71 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Whatfix</t>
+          <t>BrowserStack</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>India-HQ — Digital adoption</t>
+          <t>Mumbai / Dublin</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Remote-first (HQ Mumbai)</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Pre-IPO (secondaries on EquityZen); AE 'GTM Labs' roles OPEN now; sells US enterprise</t>
+          <t>India-HQ — Testing cloud</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Pre-IPO</t>
+          <t>Profitable; large India-based global inside-sales org; sells worldwide from India</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>AE (open now)</t>
+          <t>Profitable</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t>Competitive; pre-IPO equity</t>
+          <t>AE + SDR Manager roles recur</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>G2 DAP leader; check Glassdoor</t>
+          <t>Competitive; sales org large enough for bands</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>IPO timing uncertain</t>
+          <t>G2 strong in category</t>
         </is>
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
-          <t>Talent team via open req; VP Sales</t>
+          <t>Interview bar high; check sales Glassdoor</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr">
         <is>
-          <t>Live opening — apply + parallel warm intro</t>
-        </is>
-      </c>
-      <c r="M17" s="5" t="inlineStr">
+          <t>VP Inside Sales; Dir Sales Dev</t>
+        </is>
+      </c>
+      <c r="M17" s="4" t="inlineStr">
+        <is>
+          <t>Global-selling-from-India is their whole model</t>
+        </is>
+      </c>
+      <c r="N17" s="6" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="N17" s="5" t="n"/>
-      <c r="O17" s="5" t="n"/>
+      <c r="O17" s="6" t="n"/>
+      <c r="P17" s="6" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1669,66 +1763,71 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Mindtickle</t>
+          <t>Atlan</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Pune</t>
-        </is>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>India-HQ — Sales readiness</t>
+          <t>Delhi / Remote</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Remote-first</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Sells sales-enablement to US revenue orgs; company that trains sellers trains its own</t>
+          <t>India-HQ — Data governance</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Late-stage</t>
+          <t>$105M Series C; sells US data teams; one of strongest employer brands in Indian SaaS</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>AE; enablement-adjacent roles</t>
+          <t>Series C</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>Competitive</t>
+          <t>AE (US-facing)</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>G2 leader in sales readiness</t>
+          <t>Good; strong culture comp</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>Category consolidating</t>
+          <t>Great G2 presence; strong Glassdoor</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>VP Sales; CRO org</t>
+          <t>Data-catalog category competitive</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
         <is>
-          <t>Meta-pitch: a seller who studies selling</t>
-        </is>
-      </c>
-      <c r="M18" s="5" t="inlineStr">
+          <t>Founders; Head of Sales</t>
+        </is>
+      </c>
+      <c r="M18" s="4" t="inlineStr">
+        <is>
+          <t>Culture-first org — lead with craft and curiosity</t>
+        </is>
+      </c>
+      <c r="N18" s="6" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="N18" s="5" t="n"/>
-      <c r="O18" s="5" t="n"/>
+      <c r="O18" s="6" t="n"/>
+      <c r="P18" s="6" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1736,66 +1835,71 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Atlan</t>
+          <t>Chargebee</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Delhi / Remote</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>India-HQ — Data governance</t>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Chennai — relocation or remote exception</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>$105M Series C; sells US data teams; one of strongest employer brands in Indian SaaS</t>
+          <t>India-HQ — Billing</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>Series C</t>
+          <t>Gartner MQ Leader, Recurring Billing 2025; acquired Inai; global base sold from India</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>AE (US-facing)</t>
+          <t>Late-stage</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t>Good; strong culture comp</t>
+          <t>AE; SDR leadership</t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>Great G2 presence; strong Glassdoor</t>
+          <t>Competitive</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>Data-catalog category competitive</t>
+          <t>MQ Leader; DO the Glassdoor sales-filter check</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>Founders; Head of Sales</t>
+          <t>10% layoff late 2022</t>
         </is>
       </c>
       <c r="L19" s="4" t="inlineStr">
         <is>
-          <t>Culture-first org — lead with craft and curiosity</t>
-        </is>
-      </c>
-      <c r="M19" s="5" t="inlineStr">
+          <t>VP Sales; Dir Sales Dev</t>
+        </is>
+      </c>
+      <c r="M19" s="4" t="inlineStr">
+        <is>
+          <t>MQ Leader momentum into enterprise billing deals</t>
+        </is>
+      </c>
+      <c r="N19" s="6" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="N19" s="5" t="n"/>
-      <c r="O19" s="5" t="n"/>
+      <c r="O19" s="6" t="n"/>
+      <c r="P19" s="6" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1803,66 +1907,71 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>HighRadius</t>
+          <t>Rocketlane</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Hyderabad</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>India-HQ — Order-to-cash</t>
+          <t>Chennai</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Chennai — relocation or remote exception</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Unicorn, IPO track; large US-enterprise AE org run from Hyderabad; genuinely high OTEs</t>
+          <t>India-HQ — Onboarding/PSA</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Late-stage, IPO track</t>
+          <t>$60M Series C (Mar 2026, Insight) after doubling revenue; ex-Freshworks founders, culture reputation</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>Enterprise AE</t>
+          <t>Series C, fresh runway</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>High OTEs — among best in India</t>
+          <t>AE (high impact, small team)</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>Glassdoor polarized — talk to reps first</t>
+          <t>Mid; equity meaningful</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>High pressure; past trims</t>
+          <t>G2 momentum strong in PSA</t>
         </is>
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>VP Sales; SVP GTM</t>
+          <t>Smaller org = less structure</t>
         </is>
       </c>
       <c r="L20" s="4" t="inlineStr">
         <is>
-          <t>High-OTE enterprise seat if culture fits you</t>
-        </is>
-      </c>
-      <c r="M20" s="5" t="inlineStr">
+          <t>Founder/CEO; VP Sales</t>
+        </is>
+      </c>
+      <c r="M20" s="4" t="inlineStr">
+        <is>
+          <t>Series-C GTM expansion = they need closers now</t>
+        </is>
+      </c>
+      <c r="N20" s="6" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="N20" s="5" t="n"/>
-      <c r="O20" s="5" t="n"/>
+      <c r="O20" s="6" t="n"/>
+      <c r="P20" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1870,66 +1979,71 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>CleverTap</t>
+          <t>Darwinbox</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Mumbai</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>India-HQ — Engagement</t>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Hyderabad — relocation or remote exception</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>In Gartner 2026 MQ for personalization engines; global GTM from India</t>
+          <t>India-HQ — Enterprise HR SaaS</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
+          <t>~$300M+ raised incl. 2025; enterprise machine across India/SEA/ME/US; real enterprise ACVs</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
           <t>Late-stage</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>AE (geo pods); SDR Mgr</t>
-        </is>
-      </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t>Competitive</t>
+          <t>Enterprise AE training ground</t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>G2 solid; check Glassdoor sales</t>
+          <t>Good enterprise OTEs</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>MoEngage rivalry = market noise</t>
+          <t>Check Glassdoor sales filter</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>CRO; Regional Heads</t>
+          <t>Enterprise cycles are long; comp back-loaded</t>
         </is>
       </c>
       <c r="L21" s="4" t="inlineStr">
         <is>
-          <t>MQ placement momentum pitch</t>
-        </is>
-      </c>
-      <c r="M21" s="5" t="inlineStr">
+          <t>VP Sales (region)</t>
+        </is>
+      </c>
+      <c r="M21" s="4" t="inlineStr">
+        <is>
+          <t>Enterprise AE ambition + HR-tech domain interest</t>
+        </is>
+      </c>
+      <c r="N21" s="6" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="N21" s="5" t="n"/>
-      <c r="O21" s="5" t="n"/>
+      <c r="O21" s="6" t="n"/>
+      <c r="P21" s="6" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -1937,66 +2051,71 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>DevRev</t>
+          <t>Mindtickle</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Bengaluru + US</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>India-HQ — AI-native support/CRM</t>
+          <t>Pune</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Pune — relocation or remote exception</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>Dheeraj Pandey (Nutanix founder); heavily funded; AI-native in hot category; GTM being built</t>
+          <t>India-HQ — Sales readiness</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Well-funded, earlier GTM</t>
+          <t>Sells sales-enablement to US revenue orgs; company that trains sellers trains its own</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>Early AE (scope upside)</t>
+          <t>Late-stage</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>Mid now, equity upside</t>
+          <t>AE; enablement-adjacent roles</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>Too early for deep review data</t>
+          <t>Competitive</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>Motion still forming — risk</t>
+          <t>G2 leader in sales readiness</t>
         </is>
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
-          <t>Founder office; Head of GTM</t>
+          <t>Category consolidating</t>
         </is>
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Early-AE bet on a proven founder</t>
-        </is>
-      </c>
-      <c r="M22" s="5" t="inlineStr">
+          <t>VP Sales; CRO org</t>
+        </is>
+      </c>
+      <c r="M22" s="4" t="inlineStr">
+        <is>
+          <t>Meta-pitch: a seller who studies selling</t>
+        </is>
+      </c>
+      <c r="N22" s="6" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="N22" s="5" t="n"/>
-      <c r="O22" s="5" t="n"/>
+      <c r="O22" s="6" t="n"/>
+      <c r="P22" s="6" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -2004,66 +2123,71 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Everstage</t>
+          <t>HighRadius</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Chennai / BLR</t>
-        </is>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>India-HQ — Sales commissions</t>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>Hyderabad — relocation or remote exception</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>$44.7M raised; strong G2 momentum in incentive comp; ICP is RevOps + sales leaders</t>
+          <t>India-HQ — Order-to-cash</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>Series B</t>
+          <t>Unicorn, IPO track; large US-enterprise AE org run from Hyderabad; genuinely high OTEs</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>AE — you are the ICP</t>
+          <t>Late-stage, IPO track</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t>Mid; verify</t>
+          <t>Enterprise AE</t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>Strong G2 momentum</t>
+          <t>High OTEs — among best in India</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>Category has big incumbents (Xactly etc.)</t>
+          <t>Glassdoor polarized — talk to reps first</t>
         </is>
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
-          <t>Founder; Head of Sales</t>
+          <t>High pressure; past trims</t>
         </is>
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>A rep who lived commission pain sells this best</t>
-        </is>
-      </c>
-      <c r="M23" s="5" t="inlineStr">
+          <t>VP Sales; SVP GTM</t>
+        </is>
+      </c>
+      <c r="M23" s="4" t="inlineStr">
+        <is>
+          <t>High-OTE enterprise seat if culture fits you</t>
+        </is>
+      </c>
+      <c r="N23" s="6" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="N23" s="5" t="n"/>
-      <c r="O23" s="5" t="n"/>
+      <c r="O23" s="6" t="n"/>
+      <c r="P23" s="6" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -2071,66 +2195,71 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Amagi</t>
+          <t>CleverTap</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
-        </is>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>India-HQ — Media cloud SaaS</t>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Mumbai — relocation or remote exception</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Unicorn; turned profitable; IPO track; global media customers from India</t>
+          <t>India-HQ — Engagement</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Profitable, IPO track</t>
+          <t>In Gartner 2026 MQ for personalization engines; global GTM from India</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>AE (media vertical)</t>
+          <t>Late-stage</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
+          <t>AE (geo pods); SDR Mgr</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
           <t>Competitive</t>
         </is>
       </c>
-      <c r="I24" s="4" t="inlineStr">
-        <is>
-          <t>Check G2/Glassdoor — vertical niche</t>
-        </is>
-      </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>Vertical = narrower ICP</t>
+          <t>G2 solid; check Glassdoor sales</t>
         </is>
       </c>
       <c r="K24" s="4" t="inlineStr">
         <is>
-          <t>VP Sales</t>
+          <t>MoEngage rivalry = market noise</t>
         </is>
       </c>
       <c r="L24" s="4" t="inlineStr">
         <is>
-          <t>Vertical depth + profitability story</t>
-        </is>
-      </c>
-      <c r="M24" s="5" t="inlineStr">
+          <t>CRO; Regional Heads</t>
+        </is>
+      </c>
+      <c r="M24" s="4" t="inlineStr">
+        <is>
+          <t>MQ placement momentum pitch</t>
+        </is>
+      </c>
+      <c r="N24" s="6" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="N24" s="5" t="n"/>
-      <c r="O24" s="5" t="n"/>
+      <c r="O24" s="6" t="n"/>
+      <c r="P24" s="6" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -2146,58 +2275,63 @@
           <t>Noida / SF</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Noida — relocation or remote exception</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>India-HQ — Healthcare AI</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="F25" s="4" t="inlineStr">
         <is>
           <t>Large US healthcare sales motion supported from India; healthcare + AI double tailwind</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="G25" s="4" t="inlineStr">
         <is>
           <t>Late-stage</t>
         </is>
       </c>
-      <c r="G25" s="4" t="inlineStr">
+      <c r="H25" s="4" t="inlineStr">
         <is>
           <t>AE / sales support to US pods</t>
         </is>
       </c>
-      <c r="H25" s="4" t="inlineStr">
+      <c r="I25" s="4" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="I25" s="4" t="inlineStr">
+      <c r="J25" s="4" t="inlineStr">
         <is>
           <t>Check Glassdoor sales filter</t>
         </is>
       </c>
-      <c r="J25" s="4" t="inlineStr">
+      <c r="K25" s="4" t="inlineStr">
         <is>
           <t>US-hours overlap likely</t>
         </is>
       </c>
-      <c r="K25" s="4" t="inlineStr">
+      <c r="L25" s="4" t="inlineStr">
         <is>
           <t>GTM leadership Noida</t>
         </is>
       </c>
-      <c r="L25" s="4" t="inlineStr">
+      <c r="M25" s="4" t="inlineStr">
         <is>
           <t>Healthcare AI tailwind; India-side GTM growth</t>
         </is>
       </c>
-      <c r="M25" s="5" t="inlineStr">
+      <c r="N25" s="6" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="N25" s="5" t="n"/>
-      <c r="O25" s="5" t="n"/>
+      <c r="O25" s="6" t="n"/>
+      <c r="P25" s="6" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -2213,62 +2347,67 @@
           <t>Hyderabad</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Hyderabad — relocation or remote exception</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>India-HQ — Vertical SaaS (wellness)</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>Category leader, $1.5B val; sells US/UK from Hyderabad; has claimed profitability</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
+      <c r="G26" s="4" t="inlineStr">
         <is>
           <t>Claimed profitable</t>
         </is>
       </c>
-      <c r="G26" s="4" t="inlineStr">
+      <c r="H26" s="4" t="inlineStr">
         <is>
           <t>AE (vertical, US-facing)</t>
         </is>
       </c>
-      <c r="H26" s="4" t="inlineStr">
+      <c r="I26" s="4" t="inlineStr">
         <is>
           <t>Competitive</t>
         </is>
       </c>
-      <c r="I26" s="4" t="inlineStr">
+      <c r="J26" s="4" t="inlineStr">
         <is>
           <t>Check current Glassdoor trend</t>
         </is>
       </c>
-      <c r="J26" s="4" t="inlineStr">
+      <c r="K26" s="4" t="inlineStr">
         <is>
           <t>Last big raise 2021 — verify momentum in convo</t>
         </is>
       </c>
-      <c r="K26" s="4" t="inlineStr">
+      <c r="L26" s="4" t="inlineStr">
         <is>
           <t>VP Sales</t>
         </is>
       </c>
-      <c r="L26" s="4" t="inlineStr">
+      <c r="M26" s="4" t="inlineStr">
         <is>
           <t>Vertical leader; less competition per deal</t>
         </is>
       </c>
-      <c r="M26" s="5" t="inlineStr">
+      <c r="N26" s="6" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="N26" s="5" t="n"/>
-      <c r="O26" s="5" t="n"/>
+      <c r="O26" s="6" t="n"/>
+      <c r="P26" s="6" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="M2:M26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="N2:N26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not started,Researching,Contacted,Replied,Meeting booked,In process,Offer,Dead"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2344,12 +2483,12 @@
           <t>Huge India org, but 2026 AI-reorg layoffs hit India offices — enter with eyes open</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F2" s="5" t="n"/>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
@@ -2370,12 +2509,12 @@
           <t>Growing, big India expansion; AE seats are senior enterprise</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="n"/>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
@@ -2396,12 +2535,12 @@
           <t>High comp; sales roles competitive and process-heavy</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="n"/>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
@@ -2422,12 +2561,12 @@
           <t>Stable, strong comp; slower career velocity</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="n"/>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
@@ -2448,12 +2587,12 @@
           <t>Big India org; PIP-culture reputation in sales — check RepVue</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="n"/>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
@@ -2474,12 +2613,12 @@
           <t>Noida/Bengaluru; stable enterprise motion</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="n"/>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
@@ -2500,12 +2639,12 @@
           <t>Stable; growth flat — commissions reflect it</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="n"/>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
@@ -2526,12 +2665,12 @@
           <t>India presence; post-restructure, verify sales hiring</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="n"/>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
@@ -2552,12 +2691,12 @@
           <t>Growing security/edge play; small India GTM</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="n"/>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
@@ -2578,12 +2717,12 @@
           <t>India sales presence; solid mid-size option</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="n"/>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
@@ -2604,12 +2743,12 @@
           <t>Data streaming; India GTM exists, verify openings</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="n"/>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
@@ -2630,12 +2769,12 @@
           <t>Established India enterprise sales org</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="n"/>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
@@ -2656,12 +2795,12 @@
           <t>Stabilized after downturn; India enterprise motion</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="n"/>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
@@ -2682,12 +2821,12 @@
           <t>Security tailwind; enterprise AE seats senior</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="n"/>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
@@ -2708,12 +2847,12 @@
           <t>Security tailwind; India GTM smaller than R&amp;D</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="n"/>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
@@ -2734,12 +2873,12 @@
           <t>Largest security GTM in India of the big three</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F17" s="5" t="n"/>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
@@ -2760,12 +2899,12 @@
           <t>Identity; modest India GTM</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F18" s="5" t="n"/>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
@@ -2786,12 +2925,12 @@
           <t>Remote AEs in India; async culture</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F19" s="5" t="n"/>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
@@ -2812,12 +2951,12 @@
           <t>India GTM exists; domestic-market regulatory drag</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F20" s="5" t="n"/>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n">
@@ -2838,12 +2977,12 @@
           <t>Gurgaon GTM hub; Glassdoor mixed — check sales filter</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F21" s="5" t="n"/>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n">
@@ -2864,12 +3003,12 @@
           <t>India covered from Singapore; few India seats</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F22" s="5" t="n"/>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
@@ -2890,12 +3029,12 @@
           <t>India GTM announced; early, few sales seats</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F23" s="5" t="n"/>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n">
@@ -2916,12 +3055,12 @@
           <t>PE-owned; stable but not fast</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F24" s="5" t="n"/>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
@@ -2942,12 +3081,12 @@
           <t>Bengaluru office; small GTM — fun angle given this list</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F25" s="5" t="n"/>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
@@ -2968,12 +3107,12 @@
           <t>Very profitable, no-layoff culture; pay typically below your bar — negotiate hard</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F26" s="5" t="n"/>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
@@ -2994,12 +3133,12 @@
           <t>Chennai, profitable, calm culture</t>
         </is>
       </c>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F27" s="5" t="n"/>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
@@ -3020,12 +3159,12 @@
           <t>Profitable HR SaaS; domestic mid-market</t>
         </is>
       </c>
-      <c r="E28" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F28" s="5" t="n"/>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F28" s="6" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
@@ -3046,12 +3185,12 @@
           <t>Mumbai, bootstrapped-profitable; martech</t>
         </is>
       </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F29" s="5" t="n"/>
+      <c r="E29" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
@@ -3072,12 +3211,12 @@
           <t>Delhi, bootstrapped-profitable, global customers</t>
         </is>
       </c>
-      <c r="E30" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F30" s="5" t="n"/>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
@@ -3098,12 +3237,12 @@
           <t>Hyderabad HR SaaS; strong domestic growth</t>
         </is>
       </c>
-      <c r="E31" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F31" s="5" t="n"/>
+      <c r="E31" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
@@ -3124,12 +3263,12 @@
           <t>Unicorn; domestic-heavy; check current growth</t>
         </is>
       </c>
-      <c r="E32" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F32" s="5" t="n"/>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
@@ -3150,12 +3289,12 @@
           <t>Loyalty SaaS; IPO attempted — verify state</t>
         </is>
       </c>
-      <c r="E33" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F33" s="5" t="n"/>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
@@ -3176,12 +3315,12 @@
           <t>Profitable fintech data SaaS, IPO-bound</t>
         </is>
       </c>
-      <c r="E34" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F34" s="5" t="n"/>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
@@ -3202,12 +3341,12 @@
           <t>Identity verification; steady</t>
         </is>
       </c>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F35" s="5" t="n"/>
+      <c r="E35" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="n">
@@ -3228,12 +3367,12 @@
           <t>Chennai MSP SaaS; outbound US motion; growing</t>
         </is>
       </c>
-      <c r="E36" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F36" s="5" t="n"/>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n">
@@ -3254,12 +3393,12 @@
           <t>SaaS management; outbound US</t>
         </is>
       </c>
-      <c r="E37" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F37" s="5" t="n"/>
+      <c r="E37" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F37" s="6" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="n">
@@ -3280,12 +3419,12 @@
           <t>SaaS buying; Chennai/US</t>
         </is>
       </c>
-      <c r="E38" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F38" s="5" t="n"/>
+      <c r="E38" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n">
@@ -3306,12 +3445,12 @@
           <t>Expense management; sells US via channel</t>
         </is>
       </c>
-      <c r="E39" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F39" s="5" t="n"/>
+      <c r="E39" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="n">
@@ -3332,12 +3471,12 @@
           <t>Billing (YC); early but sharp team</t>
         </is>
       </c>
-      <c r="E40" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F40" s="5" t="n"/>
+      <c r="E40" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="n">
@@ -3358,12 +3497,12 @@
           <t>Sprinto competitor; growing</t>
         </is>
       </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F41" s="5" t="n"/>
+      <c r="E41" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="n">
@@ -3384,12 +3523,12 @@
           <t>Property ops SaaS; Chennai/NY</t>
         </is>
       </c>
-      <c r="E42" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F42" s="5" t="n"/>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="n">
@@ -3410,12 +3549,12 @@
           <t>Logistics SaaS; steady</t>
         </is>
       </c>
-      <c r="E43" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F43" s="5" t="n"/>
+      <c r="E43" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="n">
@@ -3436,12 +3575,12 @@
           <t>Logistics SaaS; Gurgaon</t>
         </is>
       </c>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F44" s="5" t="n"/>
+      <c r="E44" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="n">
@@ -3462,12 +3601,12 @@
           <t>CPaaS; profitable-ish, domestic-heavy</t>
         </is>
       </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F45" s="5" t="n"/>
+      <c r="E45" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="n">
@@ -3488,12 +3627,12 @@
           <t>Conversational messaging; profitability claimed</t>
         </is>
       </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F46" s="5" t="n"/>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n">
@@ -3514,12 +3653,12 @@
           <t>Contact-center AI; US-facing</t>
         </is>
       </c>
-      <c r="E47" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F47" s="5" t="n"/>
+      <c r="E47" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="n">
@@ -3540,12 +3679,12 @@
           <t>Conversational AI; verify momentum</t>
         </is>
       </c>
-      <c r="E48" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F48" s="5" t="n"/>
+      <c r="E48" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="4" t="n">
@@ -3566,12 +3705,12 @@
           <t>Big raises; revenue questions persist — diligence hard</t>
         </is>
       </c>
-      <c r="E49" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F49" s="5" t="n"/>
+      <c r="E49" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="4" t="n">
@@ -3592,12 +3731,12 @@
           <t>Pune CLM leader; growth slowed, still solid enterprise logo</t>
         </is>
       </c>
-      <c r="E50" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F50" s="5" t="n"/>
+      <c r="E50" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F50" s="6" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="4" t="n">
@@ -3618,12 +3757,12 @@
           <t>Pivoted to PromptQL/AI — interesting but unproven motion</t>
         </is>
       </c>
-      <c r="E51" s="5" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F51" s="5" t="n"/>
+      <c r="E51" s="6" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -3649,267 +3788,267 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>B2B SaaS Job-Search Target List — Criteria &amp; Legend</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>Built July 2026. Reference package: Rs29 LPA (comp annotated, not filtered). Target roles: SDR/BDR Manager or Account Executive.</t>
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Built July 2026. Reference package: Rs29 LPA (comp annotated, not filtered). Target roles: SDR/BDR Manager or Account Executive. Based in Bangalore — Tier 1 is sorted Bangalore-first, then remote-friendly, then relocation-required.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr"/>
+      <c r="A3" s="8" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>HOW TO USE THIS WORKBOOK</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Yellow cells are yours to edit: Status, Next Step, and My Notes columns on both target sheets.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Status column has a dropdown. Row 2 of Tier 1 (Rippling) shows example values in the yellow columns — replace them with your real progress.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Everything else is research data as of July 2026 — refresh the 'verify' items before outreach.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr"/>
+      <c r="A8" s="8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
         <is>
           <t>SELECTION SIGNALS (what each column reflects)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>Growth signal</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>GTM headcount trend, revenue growth, funding news — a company adding salespeople is one where sales is working</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>Funding / profitability</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Runway = fewer layoff surprises. Source: Tracxn, press releases</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>Reviews check</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>G2 momentum (Grid movement, review growth), Glassdoor FILTERED TO SALES DEPT, RepVue score + quota attainment</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>Risk flags</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Layoff history (18-24 mo), culture intensity, category risk</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>Role fit</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Outbound-led orgs value BDR leadership; enterprise ACV = higher OTE</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>Comp signal</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>Known ranges. Benchmarks: India AE avg ~Rs24L; top 10% &gt;Rs45L; Enterprise AE median OTE ~Rs65L (RepVue, 2026)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr"/>
+      <c r="A16" s="8" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="A17" s="8" t="inlineStr">
         <is>
           <t>15-MIN DILIGENCE BEFORE EACH OUTREACH</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>RepVue score + quota attainment (repvue.com)</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>Glassdoor filtered to sales department, last 12 months</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>LinkedIn: GTM headcount 6-month trend + average sales-rep tenure</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>Last funding round / layoffs.fyi check</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr"/>
+      <c r="A22" s="8" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="A23" s="9" t="inlineStr">
         <is>
           <t>KEY SOURCES</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="7" t="inlineStr">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>RepVue rankings &amp; salaries</t>
         </is>
       </c>
-      <c r="B24" s="7" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>repvue.com/rankings/overall ; repvue.com/salaries/account-executive/IN</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="7" t="inlineStr">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>Rippling India roles &amp; comp</t>
         </is>
       </c>
-      <c r="B25" s="7" t="inlineStr">
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>in.linkedin.com/jobs/rippling-jobs-bengaluru ; 6figr.com/in/salary/rippling</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="7" t="inlineStr">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>Rocketlane Series C (Mar 2026)</t>
         </is>
       </c>
-      <c r="B26" s="7" t="inlineStr">
+      <c r="B26" s="8" t="inlineStr">
         <is>
           <t>rocketlane.com/press/rocketlane-raises-series-c</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="inlineStr">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>MoEngage $280M Series F (Dec 2025)</t>
         </is>
       </c>
-      <c r="B27" s="7" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t>startupwired.com/2025/12/17/moengage-raises-180m-more-weeks-after-100m-funding/</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="inlineStr">
+      <c r="A28" s="8" t="inlineStr">
         <is>
           <t>Layoff trackers</t>
         </is>
       </c>
-      <c r="B28" s="7" t="inlineStr">
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t>techcrunch.com/2025/12/22/tech-layoffs-2025-list/ ; trueup.io/layoffs</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="inlineStr">
+      <c r="A29" s="8" t="inlineStr">
         <is>
           <t>India SaaS market data</t>
         </is>
       </c>
-      <c r="B29" s="7" t="inlineStr">
+      <c r="B29" s="8" t="inlineStr">
         <is>
           <t>tracxn.com — $1.26B raised across 103 rounds by Apr 2026 (+38% YoY)</t>
         </is>

</xml_diff>

<commit_message>
Rebuild tracker: leaner columns, fillable review scores, contact + last-touch tracking
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Kq1GVuDP62P4fjx7tfK9jZ
</commit_message>
<xml_diff>
--- a/outreach/target-companies-tracker.xlsx
+++ b/outreach/target-companies-tracker.xlsx
@@ -102,16 +102,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -494,25 +493,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P26"/>
+  <dimension ref="A1:R26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
     <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="30" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="26" customWidth="1" min="16" max="16"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="30" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="26" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -528,47 +529,47 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>India Hub</t>
+          <t>Location</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Bangalore Fit</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>Why It Made the List (Growth + Funding)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Why It Made the List (Growth Signal)</t>
+          <t>Role Fit</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Funding / Profitability</t>
+          <t>Comp Signal</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Role Fit</t>
+          <t>Risk Flags</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Comp Signal</t>
+          <t>RepVue Score</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Reviews Check (G2 / Glassdoor / RepVue)</t>
+          <t>Glassdoor (Sales)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Risk Flags</t>
+          <t>G2</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
@@ -578,20 +579,30 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>Contact Name / LinkedIn</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>Outreach Angle</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Last Touch</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Next Step</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>My Notes</t>
         </is>
@@ -608,72 +619,82 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
           <t>Bangalore office</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Global — HR/IT/Fin platform</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>~53 open Bengaluru roles incl. Mid-Market AE and SDR Manager (Outbound); Bangalore hub sells outbound into North America SMB/MM</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>Late-stage, hypergrowth</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>~53 open Bengaluru roles incl. Mid-Market AE and SDR Manager (Outbound); Bangalore hub sells outbound into North America SMB/MM. Late-stage, hypergrowth.</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>SDR Manager + MM AE (both open)</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>SDR median base ~Rs14L; India avg total comp ~Rs59L (6figr)</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
-        <is>
-          <t>Check RepVue + Glassdoor sales filter; strong pay reports</t>
-        </is>
-      </c>
-      <c r="K2" s="4" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Intense pace; hybrid 3 days/office; Deel litigation noise</t>
         </is>
       </c>
-      <c r="L2" s="4" t="inlineStr">
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>4.1 (example)</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>3.9 sales dept (example)</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>4.8, 3,100 reviews (example)</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Head of Sales Dev India; India GTM site lead</t>
         </is>
       </c>
-      <c r="M2" s="4" t="inlineStr">
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>e.g. Priya S — linkedin.com/in/example</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>Outbound playbook + team leadership story maps 1:1 to their outbound SMB motion</t>
         </is>
       </c>
-      <c r="N2" s="6" t="inlineStr">
+      <c r="O2" s="5" t="inlineStr">
         <is>
           <t>Contacted</t>
         </is>
       </c>
-      <c r="O2" s="6" t="inlineStr">
+      <c r="P2" s="5" t="inlineStr">
+        <is>
+          <t>21-Jul-2026</t>
+        </is>
+      </c>
+      <c r="Q2" s="5" t="inlineStr">
         <is>
           <t>Follow up 28-Jul if no reply</t>
         </is>
       </c>
-      <c r="P2" s="6" t="inlineStr">
-        <is>
-          <t>e.g. Emailed Head of Sales Dev 21-Jul via LinkedIn</t>
+      <c r="R2" s="5" t="inlineStr">
+        <is>
+          <t>Emailed Head of Sales Dev via LinkedIn</t>
         </is>
       </c>
     </row>
@@ -688,66 +709,56 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
-        </is>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
           <t>Bangalore office</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Global — Data/AI</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Among fastest-growing software cos ever; AI tailwind; 3,000+ India job listings; India-market BDR hiring seen</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>Pre-IPO, massively funded</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Among fastest-growing software cos ever; AI tailwind; 3,000+ India job listings; India-market BDR hiring seen. Pre-IPO, massively funded.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>BDR lead / commercial AE</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Top-of-market + pre-IPO equity</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>Strong employer brand; verify India sales Glassdoor</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>AE seats may be senior; India GTM younger than R&amp;D</t>
         </is>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="I3" s="5" t="n"/>
+      <c r="J3" s="5" t="n"/>
+      <c r="K3" s="5" t="n"/>
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>RVP India / India sales leadership</t>
         </is>
       </c>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="M3" s="5" t="n"/>
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>AI category momentum; ask about GTM build-out as India scales</t>
         </is>
       </c>
-      <c r="N3" s="6" t="inlineStr">
+      <c r="O3" s="5" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="O3" s="6" t="n"/>
-      <c r="P3" s="6" t="n"/>
+      <c r="P3" s="5" t="n"/>
+      <c r="Q3" s="5" t="n"/>
+      <c r="R3" s="5" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -760,66 +771,56 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Bengaluru / Mumbai</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
           <t>Bangalore office</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Global — Data cloud</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>SDR role open in Bengaluru (posted Jun 2026); public, growing, FCF positive</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>Public, profitable on FCF</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>SDR role open in Bengaluru (posted Jun 2026); public, growing, FCF positive.</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>SDR leadership path; commercial AE</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Enterprise AE OTEs high (India ent. AE median OTE ~Rs65L)</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>Solid RepVue historically</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>AE seats skew senior enterprise</t>
         </is>
       </c>
-      <c r="L4" s="4" t="inlineStr">
+      <c r="I4" s="5" t="n"/>
+      <c r="J4" s="5" t="n"/>
+      <c r="K4" s="5" t="n"/>
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t>SDR Manager India; Country Mgr</t>
         </is>
       </c>
-      <c r="M4" s="4" t="inlineStr">
+      <c r="M4" s="5" t="n"/>
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>Enterprise motion experience + outbound rigor</t>
         </is>
       </c>
-      <c r="N4" s="6" t="inlineStr">
+      <c r="O4" s="5" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="O4" s="6" t="n"/>
-      <c r="P4" s="6" t="n"/>
+      <c r="P4" s="5" t="n"/>
+      <c r="Q4" s="5" t="n"/>
+      <c r="R4" s="5" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -832,66 +833,56 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Gurgaon / Bengaluru</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
           <t>Bangalore office (verify sales seats; sales HQ Gurgaon)</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>Global — Database</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Established India-market sales org; best-known SDR-to-AE academy ladder in tech</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>Public, durable</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Established India-market sales org; best-known SDR-to-AE academy ladder in tech. Public, durable.</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>SDR Mgr or AE via ladder</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Competitive; RSUs</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
-        <is>
-          <t>Historically strong RepVue</t>
-        </is>
-      </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Growth moderated vs 2021 peaks</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="I5" s="5" t="n"/>
+      <c r="J5" s="5" t="n"/>
+      <c r="K5" s="5" t="n"/>
+      <c r="L5" s="2" t="inlineStr">
         <is>
           <t>Regional Director India</t>
         </is>
       </c>
-      <c r="M5" s="4" t="inlineStr">
+      <c r="M5" s="5" t="n"/>
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>Their promotion ladder = your AE jump story</t>
         </is>
       </c>
-      <c r="N5" s="6" t="inlineStr">
+      <c r="O5" s="5" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="O5" s="6" t="n"/>
-      <c r="P5" s="6" t="n"/>
+      <c r="P5" s="5" t="n"/>
+      <c r="Q5" s="5" t="n"/>
+      <c r="R5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -904,66 +895,56 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>India (newer)</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
           <t>Bangalore likely — verify</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Global — Observability</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>RepVue quota attainment 83.7% (elite vs ~43% industry avg); profitable, ~25% growth</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>Public, profitable</t>
-        </is>
-      </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>RepVue quota attainment 83.7% (elite vs ~43% industry avg); public, profitable, ~25% growth.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Commercial AE</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>High; verify India bands</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
-        <is>
-          <t>RepVue elite</t>
-        </is>
-      </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>India GTM footprint newer/smaller — verify openings</t>
         </is>
       </c>
-      <c r="L6" s="4" t="inlineStr">
+      <c r="I6" s="5" t="n"/>
+      <c r="J6" s="5" t="n"/>
+      <c r="K6" s="5" t="n"/>
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>APAC sales leadership</t>
         </is>
       </c>
-      <c r="M6" s="4" t="inlineStr">
+      <c r="M6" s="5" t="n"/>
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>Attainment culture pitch: you want a quota that's real</t>
         </is>
       </c>
-      <c r="N6" s="6" t="inlineStr">
+      <c r="O6" s="5" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="O6" s="6" t="n"/>
-      <c r="P6" s="6" t="n"/>
+      <c r="P6" s="5" t="n"/>
+      <c r="Q6" s="5" t="n"/>
+      <c r="R6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -976,66 +957,56 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Pune / Bengaluru</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
           <t>Bangalore office</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Global — ABM/Revenue AI</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>RepVue attainment 83.2%; large India presence; product sells to sales leaders (your persona)</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>Late-stage funded</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>RepVue attainment 83.2%; large India presence; product sells to sales leaders (your persona). Late-stage funded.</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>BDR leadership; AE (verify)</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Good; verify India bands</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr">
-        <is>
-          <t>RepVue elite</t>
-        </is>
-      </c>
-      <c r="K7" s="4" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>India roles skew R&amp;D + BDR</t>
         </is>
       </c>
-      <c r="L7" s="4" t="inlineStr">
+      <c r="I7" s="5" t="n"/>
+      <c r="J7" s="5" t="n"/>
+      <c r="K7" s="5" t="n"/>
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>India site lead; Head of SDR</t>
         </is>
       </c>
-      <c r="M7" s="4" t="inlineStr">
+      <c r="M7" s="5" t="n"/>
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>You ARE the ICP — sell sales-intelligence as a seller</t>
         </is>
       </c>
-      <c r="N7" s="6" t="inlineStr">
+      <c r="O7" s="5" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="O7" s="6" t="n"/>
-      <c r="P7" s="6" t="n"/>
+      <c r="P7" s="5" t="n"/>
+      <c r="Q7" s="5" t="n"/>
+      <c r="R7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1048,66 +1019,56 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Chennai / BLR / Hyd</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
           <t>Bangalore office (HQ Chennai)</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>India-HQ — CX/ITSM suite</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>Public; 16% YoY; EX business crossed $500M ARR; most mature sales career ladder in Indian SaaS</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>Public, strong FCF</t>
-        </is>
-      </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Public; 16% YoY; EX business crossed $500M ARR; strong FCF; most mature sales career ladder in Indian SaaS.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>SDR Mgr, AE, or Mgr track</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Competitive at senior levels; liquid RSUs</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr">
-        <is>
-          <t>G2 strong across products; filter Glassdoor to sales</t>
-        </is>
-      </c>
-      <c r="K8" s="4" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Growth moderating; Nov-2024 restructure (~13%)</t>
         </is>
       </c>
-      <c r="L8" s="4" t="inlineStr">
+      <c r="I8" s="5" t="n"/>
+      <c r="J8" s="5" t="n"/>
+      <c r="K8" s="5" t="n"/>
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>Director Sales Dev; VP Sales (segment)</t>
         </is>
       </c>
-      <c r="M8" s="4" t="inlineStr">
+      <c r="M8" s="5" t="n"/>
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>Ladder + brand; ask about MM AE or SDR leadership</t>
         </is>
       </c>
-      <c r="N8" s="6" t="inlineStr">
+      <c r="O8" s="5" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="O8" s="6" t="n"/>
-      <c r="P8" s="6" t="n"/>
+      <c r="P8" s="5" t="n"/>
+      <c r="Q8" s="5" t="n"/>
+      <c r="R8" s="5" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1120,66 +1081,56 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Bengaluru / SF</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
           <t>Bangalore office</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>India-HQ — API platform</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>$5.6B val; AI Agent momentum (Agent Builder; Fern + liblab acquisitions); moving upmarket</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>Late-stage, efficient</t>
-        </is>
-      </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>$5.6B val; AI Agent momentum (Agent Builder; Fern + liblab acquisitions); moving upmarket. Late-stage, efficient.</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Enterprise AE; sales-dev leadership</t>
         </is>
       </c>
-      <c r="I9" s="4" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Strong; equity story good</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr">
-        <is>
-          <t>G2 category leader; strong brand halo</t>
-        </is>
-      </c>
-      <c r="K9" s="4" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>PLG DNA — sales org smaller</t>
         </is>
       </c>
-      <c r="L9" s="4" t="inlineStr">
+      <c r="I9" s="5" t="n"/>
+      <c r="J9" s="5" t="n"/>
+      <c r="K9" s="5" t="n"/>
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>CRO org; Head of Enterprise Sales</t>
         </is>
       </c>
-      <c r="M9" s="4" t="inlineStr">
+      <c r="M9" s="5" t="n"/>
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>Enterprise motion is new-ish — early AE upside</t>
         </is>
       </c>
-      <c r="N9" s="6" t="inlineStr">
+      <c r="O9" s="5" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="O9" s="6" t="n"/>
-      <c r="P9" s="6" t="n"/>
+      <c r="P9" s="5" t="n"/>
+      <c r="Q9" s="5" t="n"/>
+      <c r="R9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -1192,66 +1143,56 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
           <t>Bangalore HQ (remote-first)</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>India-HQ — Compliance automation</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>~$38M ARR compounding; outbound-heavy US SMB/MM motion — most BDR-manager-shaped org on list</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>Series B, efficient</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>~$38M ARR compounding; outbound-heavy US SMB/MM motion — most BDR-manager-shaped org on list; strong G2 vs Vanta/Drata. Series B, efficient.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>SDR/BDR Manager (ideal); AE</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Mid-to-good; verify OTE split</t>
         </is>
       </c>
-      <c r="J10" s="4" t="inlineStr">
-        <is>
-          <t>G2 strong vs Vanta/Drata</t>
-        </is>
-      </c>
-      <c r="K10" s="4" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>Earlier stage; check attainment claims</t>
         </is>
       </c>
-      <c r="L10" s="4" t="inlineStr">
+      <c r="I10" s="5" t="n"/>
+      <c r="J10" s="5" t="n"/>
+      <c r="K10" s="5" t="n"/>
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>Founder; Head of Sales</t>
         </is>
       </c>
-      <c r="M10" s="4" t="inlineStr">
+      <c r="M10" s="5" t="n"/>
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>Outbound org needs outbound leadership — direct fit</t>
         </is>
       </c>
-      <c r="N10" s="6" t="inlineStr">
+      <c r="O10" s="5" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="O10" s="6" t="n"/>
-      <c r="P10" s="6" t="n"/>
+      <c r="P10" s="5" t="n"/>
+      <c r="Q10" s="5" t="n"/>
+      <c r="R10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1264,66 +1205,56 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
           <t>Bangalore HQ</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>India-HQ — Customer engagement</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>~$280M Series F (Dec 2025) — explicit GTM war chest; US/EU/SEA expansion</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>Series F, funded for GTM</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>~$280M Series F (Dec 2025) — explicit GTM war chest; US/EU/SEA expansion from India.</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>AE (multiple geos); SDR Mgr</t>
         </is>
       </c>
-      <c r="I11" s="4" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Competitive post-raise</t>
         </is>
       </c>
-      <c r="J11" s="4" t="inlineStr">
-        <is>
-          <t>G2 solid; check Glassdoor sales</t>
-        </is>
-      </c>
-      <c r="K11" s="4" t="inlineStr">
-        <is>
-          <t>Integration of big raise = org churn possible</t>
-        </is>
-      </c>
-      <c r="L11" s="4" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Big-raise integration = possible org churn</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="n"/>
+      <c r="J11" s="5" t="n"/>
+      <c r="K11" s="5" t="n"/>
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>CRO; Regional VPs</t>
         </is>
       </c>
-      <c r="M11" s="4" t="inlineStr">
+      <c r="M11" s="5" t="n"/>
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>Fresh capital earmarked for GTM = hiring wave</t>
         </is>
       </c>
-      <c r="N11" s="6" t="inlineStr">
+      <c r="O11" s="5" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="O11" s="6" t="n"/>
-      <c r="P11" s="6" t="n"/>
+      <c r="P11" s="5" t="n"/>
+      <c r="Q11" s="5" t="n"/>
+      <c r="R11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1336,66 +1267,56 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
           <t>Bangalore HQ</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>India-HQ — Digital adoption</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>Pre-IPO (secondaries on EquityZen); AE 'GTM Labs' roles OPEN now; sells US enterprise</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>Pre-IPO</t>
-        </is>
-      </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Pre-IPO (secondaries on EquityZen); AE 'GTM Labs' roles OPEN now; sells US enterprise; G2 DAP leader.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>AE (open now)</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Competitive; pre-IPO equity</t>
         </is>
       </c>
-      <c r="J12" s="4" t="inlineStr">
-        <is>
-          <t>G2 DAP leader; check Glassdoor</t>
-        </is>
-      </c>
-      <c r="K12" s="4" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>IPO timing uncertain</t>
         </is>
       </c>
-      <c r="L12" s="4" t="inlineStr">
+      <c r="I12" s="5" t="n"/>
+      <c r="J12" s="5" t="n"/>
+      <c r="K12" s="5" t="n"/>
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>Talent team via open req; VP Sales</t>
         </is>
       </c>
-      <c r="M12" s="4" t="inlineStr">
+      <c r="M12" s="5" t="n"/>
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>Live opening — apply + parallel warm intro</t>
         </is>
       </c>
-      <c r="N12" s="6" t="inlineStr">
+      <c r="O12" s="5" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="O12" s="6" t="n"/>
-      <c r="P12" s="6" t="n"/>
+      <c r="P12" s="5" t="n"/>
+      <c r="Q12" s="5" t="n"/>
+      <c r="R12" s="5" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1408,66 +1329,56 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Bengaluru + US</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
           <t>Bangalore office</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>India-HQ — AI-native support/CRM</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>Dheeraj Pandey (Nutanix founder); heavily funded; AI-native in hot category; GTM being built</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>Well-funded, earlier GTM</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Dheeraj Pandey (Nutanix founder); heavily funded; AI-native in hot category; GTM being built.</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Early AE (scope upside)</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Mid now, equity upside</t>
         </is>
       </c>
-      <c r="J13" s="4" t="inlineStr">
-        <is>
-          <t>Too early for deep review data</t>
-        </is>
-      </c>
-      <c r="K13" s="4" t="inlineStr">
-        <is>
-          <t>Motion still forming — risk</t>
-        </is>
-      </c>
-      <c r="L13" s="4" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Motion still forming — earlier-stage risk</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="n"/>
+      <c r="J13" s="5" t="n"/>
+      <c r="K13" s="5" t="n"/>
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>Founder office; Head of GTM</t>
         </is>
       </c>
-      <c r="M13" s="4" t="inlineStr">
+      <c r="M13" s="5" t="n"/>
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>Early-AE bet on a proven founder</t>
         </is>
       </c>
-      <c r="N13" s="6" t="inlineStr">
+      <c r="O13" s="5" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="O13" s="6" t="n"/>
-      <c r="P13" s="6" t="n"/>
+      <c r="P13" s="5" t="n"/>
+      <c r="Q13" s="5" t="n"/>
+      <c r="R13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1480,66 +1391,56 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Chennai / BLR</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
           <t>Bangalore presence (HQ Chennai)</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>India-HQ — Sales commissions</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>$44.7M raised; strong G2 momentum in incentive comp; ICP is RevOps + sales leaders</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>Series B</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>$44.7M raised; strong G2 momentum in incentive comp; ICP is RevOps + sales leaders. Series B.</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>AE — you are the ICP</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>Mid; verify</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr">
-        <is>
-          <t>Strong G2 momentum</t>
-        </is>
-      </c>
-      <c r="K14" s="4" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Category has big incumbents (Xactly etc.)</t>
         </is>
       </c>
-      <c r="L14" s="4" t="inlineStr">
+      <c r="I14" s="5" t="n"/>
+      <c r="J14" s="5" t="n"/>
+      <c r="K14" s="5" t="n"/>
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t>Founder; Head of Sales</t>
         </is>
       </c>
-      <c r="M14" s="4" t="inlineStr">
+      <c r="M14" s="5" t="n"/>
+      <c r="N14" s="2" t="inlineStr">
         <is>
           <t>A rep who lived commission pain sells this best</t>
         </is>
       </c>
-      <c r="N14" s="6" t="inlineStr">
+      <c r="O14" s="5" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="O14" s="6" t="n"/>
-      <c r="P14" s="6" t="n"/>
+      <c r="P14" s="5" t="n"/>
+      <c r="Q14" s="5" t="n"/>
+      <c r="R14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1552,66 +1453,56 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Bengaluru</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
           <t>Bangalore HQ</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>India-HQ — Media cloud SaaS</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>Unicorn; turned profitable; IPO track; global media customers from India</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>Profitable, IPO track</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Unicorn; turned profitable; IPO track; global media customers from India.</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>AE (media vertical)</t>
         </is>
       </c>
-      <c r="I15" s="4" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>Competitive</t>
         </is>
       </c>
-      <c r="J15" s="4" t="inlineStr">
-        <is>
-          <t>Check G2/Glassdoor — vertical niche</t>
-        </is>
-      </c>
-      <c r="K15" s="4" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>Vertical = narrower ICP</t>
         </is>
       </c>
-      <c r="L15" s="4" t="inlineStr">
+      <c r="I15" s="5" t="n"/>
+      <c r="J15" s="5" t="n"/>
+      <c r="K15" s="5" t="n"/>
+      <c r="L15" s="2" t="inlineStr">
         <is>
           <t>VP Sales</t>
         </is>
       </c>
-      <c r="M15" s="4" t="inlineStr">
+      <c r="M15" s="5" t="n"/>
+      <c r="N15" s="2" t="inlineStr">
         <is>
           <t>Vertical depth + profitability story</t>
         </is>
       </c>
-      <c r="N15" s="6" t="inlineStr">
+      <c r="O15" s="5" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="O15" s="6" t="n"/>
-      <c r="P15" s="6" t="n"/>
+      <c r="P15" s="5" t="n"/>
+      <c r="Q15" s="5" t="n"/>
+      <c r="R15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1627,63 +1518,53 @@
           <t>Remote (India)</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>Remote (India)</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>Global — Payroll/EOR</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>~$1B ARR, profitable; hires remote AEs/SDR leaders in India timezones for APAC/EMEA</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>Profitable</t>
-        </is>
-      </c>
-      <c r="H16" s="4" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>~$1B ARR, profitable; hires remote AEs/SDR leaders in India timezones for APAC/EMEA.</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Remote AE / SDR leader</t>
         </is>
       </c>
-      <c r="I16" s="4" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>Strong global-remote bands</t>
         </is>
       </c>
-      <c r="J16" s="4" t="inlineStr">
-        <is>
-          <t>Check RepVue; fast-paced</t>
-        </is>
-      </c>
-      <c r="K16" s="4" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>Fully remote culture; Rippling feud</t>
         </is>
       </c>
-      <c r="L16" s="4" t="inlineStr">
+      <c r="I16" s="5" t="n"/>
+      <c r="J16" s="5" t="n"/>
+      <c r="K16" s="5" t="n"/>
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>APAC sales leadership</t>
         </is>
       </c>
-      <c r="M16" s="4" t="inlineStr">
+      <c r="M16" s="5" t="n"/>
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>Remote + APAC coverage experience</t>
         </is>
       </c>
-      <c r="N16" s="6" t="inlineStr">
+      <c r="O16" s="5" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="O16" s="6" t="n"/>
-      <c r="P16" s="6" t="n"/>
+      <c r="P16" s="5" t="n"/>
+      <c r="Q16" s="5" t="n"/>
+      <c r="R16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1696,66 +1577,56 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Mumbai / Dublin</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
           <t>Remote-first (HQ Mumbai)</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>India-HQ — Testing cloud</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>Profitable; large India-based global inside-sales org; sells worldwide from India</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>Profitable</t>
-        </is>
-      </c>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Profitable; large India-based global inside-sales org; sells worldwide from India; strong G2 in category.</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>AE + SDR Manager roles recur</t>
         </is>
       </c>
-      <c r="I17" s="4" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>Competitive; sales org large enough for bands</t>
         </is>
       </c>
-      <c r="J17" s="4" t="inlineStr">
-        <is>
-          <t>G2 strong in category</t>
-        </is>
-      </c>
-      <c r="K17" s="4" t="inlineStr">
-        <is>
-          <t>Interview bar high; check sales Glassdoor</t>
-        </is>
-      </c>
-      <c r="L17" s="4" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Interview bar high</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="n"/>
+      <c r="J17" s="5" t="n"/>
+      <c r="K17" s="5" t="n"/>
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>VP Inside Sales; Dir Sales Dev</t>
         </is>
       </c>
-      <c r="M17" s="4" t="inlineStr">
+      <c r="M17" s="5" t="n"/>
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>Global-selling-from-India is their whole model</t>
         </is>
       </c>
-      <c r="N17" s="6" t="inlineStr">
+      <c r="O17" s="5" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="O17" s="6" t="n"/>
-      <c r="P17" s="6" t="n"/>
+      <c r="P17" s="5" t="n"/>
+      <c r="Q17" s="5" t="n"/>
+      <c r="R17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1768,66 +1639,56 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Delhi / Remote</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
           <t>Remote-first</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>India-HQ — Data governance</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>$105M Series C; sells US data teams; one of strongest employer brands in Indian SaaS</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>Series C</t>
-        </is>
-      </c>
-      <c r="H18" s="4" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>$105M Series C; sells US data teams; one of strongest employer brands in Indian SaaS.</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>AE (US-facing)</t>
         </is>
       </c>
-      <c r="I18" s="4" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Good; strong culture comp</t>
         </is>
       </c>
-      <c r="J18" s="4" t="inlineStr">
-        <is>
-          <t>Great G2 presence; strong Glassdoor</t>
-        </is>
-      </c>
-      <c r="K18" s="4" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>Data-catalog category competitive</t>
         </is>
       </c>
-      <c r="L18" s="4" t="inlineStr">
+      <c r="I18" s="5" t="n"/>
+      <c r="J18" s="5" t="n"/>
+      <c r="K18" s="5" t="n"/>
+      <c r="L18" s="2" t="inlineStr">
         <is>
           <t>Founders; Head of Sales</t>
         </is>
       </c>
-      <c r="M18" s="4" t="inlineStr">
+      <c r="M18" s="5" t="n"/>
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>Culture-first org — lead with craft and curiosity</t>
         </is>
       </c>
-      <c r="N18" s="6" t="inlineStr">
+      <c r="O18" s="5" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="O18" s="6" t="n"/>
-      <c r="P18" s="6" t="n"/>
+      <c r="P18" s="5" t="n"/>
+      <c r="Q18" s="5" t="n"/>
+      <c r="R18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1840,66 +1701,56 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Chennai</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
           <t>Chennai — relocation or remote exception</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>India-HQ — Billing</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>Gartner MQ Leader, Recurring Billing 2025; acquired Inai; global base sold from India</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>Late-stage</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Gartner MQ Leader, Recurring Billing 2025; acquired Inai; global base sold from India. Late-stage.</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>AE; SDR leadership</t>
         </is>
       </c>
-      <c r="I19" s="4" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>Competitive</t>
         </is>
       </c>
-      <c r="J19" s="4" t="inlineStr">
-        <is>
-          <t>MQ Leader; DO the Glassdoor sales-filter check</t>
-        </is>
-      </c>
-      <c r="K19" s="4" t="inlineStr">
-        <is>
-          <t>10% layoff late 2022</t>
-        </is>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>10% layoff late 2022 — check Glassdoor sales filter</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="n"/>
+      <c r="J19" s="5" t="n"/>
+      <c r="K19" s="5" t="n"/>
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>VP Sales; Dir Sales Dev</t>
         </is>
       </c>
-      <c r="M19" s="4" t="inlineStr">
+      <c r="M19" s="5" t="n"/>
+      <c r="N19" s="2" t="inlineStr">
         <is>
           <t>MQ Leader momentum into enterprise billing deals</t>
         </is>
       </c>
-      <c r="N19" s="6" t="inlineStr">
+      <c r="O19" s="5" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="O19" s="6" t="n"/>
-      <c r="P19" s="6" t="n"/>
+      <c r="P19" s="5" t="n"/>
+      <c r="Q19" s="5" t="n"/>
+      <c r="R19" s="5" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1912,66 +1763,56 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Chennai</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
           <t>Chennai — relocation or remote exception</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>India-HQ — Onboarding/PSA</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>$60M Series C (Mar 2026, Insight) after doubling revenue; ex-Freshworks founders, culture reputation</t>
-        </is>
-      </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>Series C, fresh runway</t>
-        </is>
-      </c>
-      <c r="H20" s="4" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>$60M Series C (Mar 2026, Insight) after doubling revenue; ex-Freshworks founders, culture reputation; strong G2 in PSA.</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>AE (high impact, small team)</t>
         </is>
       </c>
-      <c r="I20" s="4" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>Mid; equity meaningful</t>
         </is>
       </c>
-      <c r="J20" s="4" t="inlineStr">
-        <is>
-          <t>G2 momentum strong in PSA</t>
-        </is>
-      </c>
-      <c r="K20" s="4" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>Smaller org = less structure</t>
         </is>
       </c>
-      <c r="L20" s="4" t="inlineStr">
+      <c r="I20" s="5" t="n"/>
+      <c r="J20" s="5" t="n"/>
+      <c r="K20" s="5" t="n"/>
+      <c r="L20" s="2" t="inlineStr">
         <is>
           <t>Founder/CEO; VP Sales</t>
         </is>
       </c>
-      <c r="M20" s="4" t="inlineStr">
+      <c r="M20" s="5" t="n"/>
+      <c r="N20" s="2" t="inlineStr">
         <is>
           <t>Series-C GTM expansion = they need closers now</t>
         </is>
       </c>
-      <c r="N20" s="6" t="inlineStr">
+      <c r="O20" s="5" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="O20" s="6" t="n"/>
-      <c r="P20" s="6" t="n"/>
+      <c r="P20" s="5" t="n"/>
+      <c r="Q20" s="5" t="n"/>
+      <c r="R20" s="5" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1984,66 +1825,56 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Hyderabad</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
           <t>Hyderabad — relocation or remote exception</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>India-HQ — Enterprise HR SaaS</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>~$300M+ raised incl. 2025; enterprise machine across India/SEA/ME/US; real enterprise ACVs</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>Late-stage</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>~$300M+ raised incl. 2025; enterprise machine across India/SEA/ME/US; real enterprise ACVs. Late-stage.</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>Enterprise AE training ground</t>
         </is>
       </c>
-      <c r="I21" s="4" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>Good enterprise OTEs</t>
         </is>
       </c>
-      <c r="J21" s="4" t="inlineStr">
-        <is>
-          <t>Check Glassdoor sales filter</t>
-        </is>
-      </c>
-      <c r="K21" s="4" t="inlineStr">
-        <is>
-          <t>Enterprise cycles are long; comp back-loaded</t>
-        </is>
-      </c>
-      <c r="L21" s="4" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Enterprise cycles long; comp back-loaded</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="n"/>
+      <c r="J21" s="5" t="n"/>
+      <c r="K21" s="5" t="n"/>
+      <c r="L21" s="2" t="inlineStr">
         <is>
           <t>VP Sales (region)</t>
         </is>
       </c>
-      <c r="M21" s="4" t="inlineStr">
+      <c r="M21" s="5" t="n"/>
+      <c r="N21" s="2" t="inlineStr">
         <is>
           <t>Enterprise AE ambition + HR-tech domain interest</t>
         </is>
       </c>
-      <c r="N21" s="6" t="inlineStr">
+      <c r="O21" s="5" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="O21" s="6" t="n"/>
-      <c r="P21" s="6" t="n"/>
+      <c r="P21" s="5" t="n"/>
+      <c r="Q21" s="5" t="n"/>
+      <c r="R21" s="5" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -2056,66 +1887,56 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Pune</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
           <t>Pune — relocation or remote exception</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>India-HQ — Sales readiness</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>Sells sales-enablement to US revenue orgs; company that trains sellers trains its own</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>Late-stage</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Sells sales-enablement to US revenue orgs; G2 leader in sales readiness. Late-stage.</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>AE; enablement-adjacent roles</t>
         </is>
       </c>
-      <c r="I22" s="4" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>Competitive</t>
         </is>
       </c>
-      <c r="J22" s="4" t="inlineStr">
-        <is>
-          <t>G2 leader in sales readiness</t>
-        </is>
-      </c>
-      <c r="K22" s="4" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>Category consolidating</t>
         </is>
       </c>
-      <c r="L22" s="4" t="inlineStr">
+      <c r="I22" s="5" t="n"/>
+      <c r="J22" s="5" t="n"/>
+      <c r="K22" s="5" t="n"/>
+      <c r="L22" s="2" t="inlineStr">
         <is>
           <t>VP Sales; CRO org</t>
         </is>
       </c>
-      <c r="M22" s="4" t="inlineStr">
+      <c r="M22" s="5" t="n"/>
+      <c r="N22" s="2" t="inlineStr">
         <is>
           <t>Meta-pitch: a seller who studies selling</t>
         </is>
       </c>
-      <c r="N22" s="6" t="inlineStr">
+      <c r="O22" s="5" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="O22" s="6" t="n"/>
-      <c r="P22" s="6" t="n"/>
+      <c r="P22" s="5" t="n"/>
+      <c r="Q22" s="5" t="n"/>
+      <c r="R22" s="5" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -2128,66 +1949,56 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Hyderabad</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
           <t>Hyderabad — relocation or remote exception</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>India-HQ — Order-to-cash</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>Unicorn, IPO track; large US-enterprise AE org run from Hyderabad; genuinely high OTEs</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>Late-stage, IPO track</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Unicorn, IPO track; large US-enterprise AE org run from Hyderabad; genuinely high OTEs.</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>Enterprise AE</t>
         </is>
       </c>
-      <c r="I23" s="4" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>High OTEs — among best in India</t>
         </is>
       </c>
-      <c r="J23" s="4" t="inlineStr">
-        <is>
-          <t>Glassdoor polarized — talk to reps first</t>
-        </is>
-      </c>
-      <c r="K23" s="4" t="inlineStr">
-        <is>
-          <t>High pressure; past trims</t>
-        </is>
-      </c>
-      <c r="L23" s="4" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Glassdoor polarized; high pressure; past trims — talk to reps first</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="n"/>
+      <c r="J23" s="5" t="n"/>
+      <c r="K23" s="5" t="n"/>
+      <c r="L23" s="2" t="inlineStr">
         <is>
           <t>VP Sales; SVP GTM</t>
         </is>
       </c>
-      <c r="M23" s="4" t="inlineStr">
+      <c r="M23" s="5" t="n"/>
+      <c r="N23" s="2" t="inlineStr">
         <is>
           <t>High-OTE enterprise seat if culture fits you</t>
         </is>
       </c>
-      <c r="N23" s="6" t="inlineStr">
+      <c r="O23" s="5" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="O23" s="6" t="n"/>
-      <c r="P23" s="6" t="n"/>
+      <c r="P23" s="5" t="n"/>
+      <c r="Q23" s="5" t="n"/>
+      <c r="R23" s="5" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -2200,66 +2011,56 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Mumbai</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
           <t>Mumbai — relocation or remote exception</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>India-HQ — Engagement</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>In Gartner 2026 MQ for personalization engines; global GTM from India</t>
-        </is>
-      </c>
-      <c r="G24" s="4" t="inlineStr">
-        <is>
-          <t>Late-stage</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>In Gartner 2026 MQ for personalization engines; global GTM from India. Late-stage.</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>AE (geo pods); SDR Mgr</t>
         </is>
       </c>
-      <c r="I24" s="4" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>Competitive</t>
         </is>
       </c>
-      <c r="J24" s="4" t="inlineStr">
-        <is>
-          <t>G2 solid; check Glassdoor sales</t>
-        </is>
-      </c>
-      <c r="K24" s="4" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>MoEngage rivalry = market noise</t>
         </is>
       </c>
-      <c r="L24" s="4" t="inlineStr">
+      <c r="I24" s="5" t="n"/>
+      <c r="J24" s="5" t="n"/>
+      <c r="K24" s="5" t="n"/>
+      <c r="L24" s="2" t="inlineStr">
         <is>
           <t>CRO; Regional Heads</t>
         </is>
       </c>
-      <c r="M24" s="4" t="inlineStr">
+      <c r="M24" s="5" t="n"/>
+      <c r="N24" s="2" t="inlineStr">
         <is>
           <t>MQ placement momentum pitch</t>
         </is>
       </c>
-      <c r="N24" s="6" t="inlineStr">
+      <c r="O24" s="5" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="O24" s="6" t="n"/>
-      <c r="P24" s="6" t="n"/>
+      <c r="P24" s="5" t="n"/>
+      <c r="Q24" s="5" t="n"/>
+      <c r="R24" s="5" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -2272,66 +2073,56 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Noida / SF</t>
-        </is>
-      </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
           <t>Noida — relocation or remote exception</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>India-HQ — Healthcare AI</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
-        <is>
-          <t>Large US healthcare sales motion supported from India; healthcare + AI double tailwind</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>Late-stage</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Large US healthcare sales motion supported from India; well funded; healthcare + AI double tailwind.</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
         <is>
           <t>AE / sales support to US pods</t>
         </is>
       </c>
-      <c r="I25" s="4" t="inlineStr">
+      <c r="G25" s="2" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="J25" s="4" t="inlineStr">
-        <is>
-          <t>Check Glassdoor sales filter</t>
-        </is>
-      </c>
-      <c r="K25" s="4" t="inlineStr">
+      <c r="H25" s="2" t="inlineStr">
         <is>
           <t>US-hours overlap likely</t>
         </is>
       </c>
-      <c r="L25" s="4" t="inlineStr">
+      <c r="I25" s="5" t="n"/>
+      <c r="J25" s="5" t="n"/>
+      <c r="K25" s="5" t="n"/>
+      <c r="L25" s="2" t="inlineStr">
         <is>
           <t>GTM leadership Noida</t>
         </is>
       </c>
-      <c r="M25" s="4" t="inlineStr">
+      <c r="M25" s="5" t="n"/>
+      <c r="N25" s="2" t="inlineStr">
         <is>
           <t>Healthcare AI tailwind; India-side GTM growth</t>
         </is>
       </c>
-      <c r="N25" s="6" t="inlineStr">
+      <c r="O25" s="5" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="O25" s="6" t="n"/>
-      <c r="P25" s="6" t="n"/>
+      <c r="P25" s="5" t="n"/>
+      <c r="Q25" s="5" t="n"/>
+      <c r="R25" s="5" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -2344,70 +2135,60 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Hyderabad</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
           <t>Hyderabad — relocation or remote exception</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>India-HQ — Vertical SaaS (wellness)</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
-        <is>
-          <t>Category leader, $1.5B val; sells US/UK from Hyderabad; has claimed profitability</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>Claimed profitable</t>
-        </is>
-      </c>
-      <c r="H26" s="4" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Category leader, $1.5B val; sells US/UK from Hyderabad; has claimed profitability.</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>AE (vertical, US-facing)</t>
         </is>
       </c>
-      <c r="I26" s="4" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>Competitive</t>
         </is>
       </c>
-      <c r="J26" s="4" t="inlineStr">
-        <is>
-          <t>Check current Glassdoor trend</t>
-        </is>
-      </c>
-      <c r="K26" s="4" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>Last big raise 2021 — verify momentum in convo</t>
         </is>
       </c>
-      <c r="L26" s="4" t="inlineStr">
+      <c r="I26" s="5" t="n"/>
+      <c r="J26" s="5" t="n"/>
+      <c r="K26" s="5" t="n"/>
+      <c r="L26" s="2" t="inlineStr">
         <is>
           <t>VP Sales</t>
         </is>
       </c>
-      <c r="M26" s="4" t="inlineStr">
+      <c r="M26" s="5" t="n"/>
+      <c r="N26" s="2" t="inlineStr">
         <is>
           <t>Vertical leader; less competition per deal</t>
         </is>
       </c>
-      <c r="N26" s="6" t="inlineStr">
+      <c r="O26" s="5" t="inlineStr">
         <is>
           <t>Not started</t>
         </is>
       </c>
-      <c r="O26" s="6" t="n"/>
-      <c r="P26" s="6" t="n"/>
+      <c r="P26" s="5" t="n"/>
+      <c r="Q26" s="5" t="n"/>
+      <c r="R26" s="5" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="N2:N26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="O2:O26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not started,Researching,Contacted,Replied,Meeting booked,In process,Offer,Dead"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2465,7 +2246,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="n">
+      <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -2473,25 +2254,25 @@
           <t>Salesforce</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Global majors</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Huge India org, but 2026 AI-reorg layoffs hit India offices — enter with eyes open</t>
         </is>
       </c>
-      <c r="E2" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F2" s="6" t="n"/>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="n">
+      <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -2499,25 +2280,25 @@
           <t>ServiceNow</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Global majors</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Growing, big India expansion; AE seats are senior enterprise</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F3" s="6" t="n"/>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="n">
+      <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -2525,25 +2306,25 @@
           <t>Google Cloud</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Global majors</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>High comp; sales roles competitive and process-heavy</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="n"/>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="n">
+      <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -2551,25 +2332,25 @@
           <t>Microsoft</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Global majors</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>Stable, strong comp; slower career velocity</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="n"/>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="n">
+      <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -2577,25 +2358,25 @@
           <t>AWS</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Global majors</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Big India org; PIP-culture reputation in sales — check RepVue</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="n"/>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="n">
+      <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -2603,25 +2384,25 @@
           <t>Adobe (DX)</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Global majors</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Noida/Bengaluru; stable enterprise motion</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="n"/>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="n">
+      <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -2629,25 +2410,25 @@
           <t>Zoom</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Global majors</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>Stable; growth flat — commissions reflect it</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="n"/>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="n">
+      <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -2655,25 +2436,25 @@
           <t>Twilio</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Global majors</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>India presence; post-restructure, verify sales hiring</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="n"/>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="n">
+      <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -2681,25 +2462,25 @@
           <t>Cloudflare</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Global majors</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>Growing security/edge play; small India GTM</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="n"/>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="n">
+      <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -2707,25 +2488,25 @@
           <t>Elastic</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Global majors</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>India sales presence; solid mid-size option</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="n"/>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="n">
+      <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -2733,25 +2514,25 @@
           <t>Confluent</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Global majors</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>Data streaming; India GTM exists, verify openings</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="n"/>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="n">
+      <c r="A13" s="2" t="n">
         <v>12</v>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -2759,25 +2540,25 @@
           <t>Nutanix</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Global majors</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>Established India enterprise sales org</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="n"/>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="n">
+      <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -2785,25 +2566,25 @@
           <t>UiPath</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>Global majors</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>Stabilized after downturn; India enterprise motion</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="n"/>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="n">
+      <c r="A15" s="2" t="n">
         <v>14</v>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -2811,25 +2592,25 @@
           <t>Zscaler</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="2" t="inlineStr">
         <is>
           <t>Global majors</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>Security tailwind; enterprise AE seats senior</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="n"/>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="n">
+      <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -2837,25 +2618,25 @@
           <t>CrowdStrike</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Global majors</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>Security tailwind; India GTM smaller than R&amp;D</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="n"/>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="n">
+      <c r="A17" s="2" t="n">
         <v>16</v>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -2863,25 +2644,25 @@
           <t>Palo Alto Networks</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>Global majors</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>Largest security GTM in India of the big three</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="n"/>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="n">
+      <c r="A18" s="2" t="n">
         <v>17</v>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -2889,25 +2670,25 @@
           <t>Okta</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>Global majors</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>Identity; modest India GTM</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="n"/>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="n">
+      <c r="A19" s="2" t="n">
         <v>18</v>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -2915,25 +2696,25 @@
           <t>GitLab</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Global majors</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>Remote AEs in India; async culture</t>
         </is>
       </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="n"/>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="n">
+      <c r="A20" s="2" t="n">
         <v>19</v>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -2941,25 +2722,25 @@
           <t>Stripe</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>Global majors</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>India GTM exists; domestic-market regulatory drag</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="n"/>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="n">
+      <c r="A21" s="2" t="n">
         <v>20</v>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -2967,25 +2748,25 @@
           <t>Sprinklr</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>Global majors</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>Gurgaon GTM hub; Glassdoor mixed — check sales filter</t>
         </is>
       </c>
-      <c r="E21" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="n"/>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="n">
+      <c r="A22" s="2" t="n">
         <v>21</v>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -2993,25 +2774,25 @@
           <t>HubSpot</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>Global majors</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>India covered from Singapore; few India seats</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="n"/>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="n">
+      <c r="A23" s="2" t="n">
         <v>22</v>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -3019,25 +2800,25 @@
           <t>Canva</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>Global majors</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>India GTM announced; early, few sales seats</t>
         </is>
       </c>
-      <c r="E23" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F23" s="6" t="n"/>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="n">
+      <c r="A24" s="2" t="n">
         <v>23</v>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -3045,25 +2826,25 @@
           <t>Zendesk</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>Global majors</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>PE-owned; stable but not fast</t>
         </is>
       </c>
-      <c r="E24" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="n"/>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="n">
+      <c r="A25" s="2" t="n">
         <v>24</v>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -3071,25 +2852,25 @@
           <t>G2</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>Global majors</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>Bengaluru office; small GTM — fun angle given this list</t>
         </is>
       </c>
-      <c r="E25" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="n"/>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="n">
+      <c r="A26" s="2" t="n">
         <v>25</v>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -3097,25 +2878,25 @@
           <t>Zoho</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>India profitable</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>Very profitable, no-layoff culture; pay typically below your bar — negotiate hard</t>
         </is>
       </c>
-      <c r="E26" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="n"/>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="n">
+      <c r="A27" s="2" t="n">
         <v>26</v>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -3123,25 +2904,25 @@
           <t>Kissflow</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>India profitable</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>Chennai, profitable, calm culture</t>
         </is>
       </c>
-      <c r="E27" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="n"/>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="n">
+      <c r="A28" s="2" t="n">
         <v>27</v>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -3149,25 +2930,25 @@
           <t>greytHR</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>India profitable</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>Profitable HR SaaS; domestic mid-market</t>
         </is>
       </c>
-      <c r="E28" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="n"/>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="n">
+      <c r="A29" s="2" t="n">
         <v>28</v>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -3175,25 +2956,25 @@
           <t>Netcore</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>India profitable</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>Mumbai, bootstrapped-profitable; martech</t>
         </is>
       </c>
-      <c r="E29" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F29" s="6" t="n"/>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="n">
+      <c r="A30" s="2" t="n">
         <v>29</v>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -3201,25 +2982,25 @@
           <t>Wingify (VWO)</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>India profitable</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>Delhi, bootstrapped-profitable, global customers</t>
         </is>
       </c>
-      <c r="E30" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="n"/>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="n">
+      <c r="A31" s="2" t="n">
         <v>30</v>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -3227,25 +3008,25 @@
           <t>Keka</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>India profitable</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>Hyderabad HR SaaS; strong domestic growth</t>
         </is>
       </c>
-      <c r="E31" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F31" s="6" t="n"/>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="n">
+      <c r="A32" s="2" t="n">
         <v>31</v>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -3253,25 +3034,25 @@
           <t>LeadSquared</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>India profitable</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>Unicorn; domestic-heavy; check current growth</t>
         </is>
       </c>
-      <c r="E32" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="n"/>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="n">
+      <c r="A33" s="2" t="n">
         <v>32</v>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -3279,25 +3060,25 @@
           <t>Capillary</t>
         </is>
       </c>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>India profitable</t>
         </is>
       </c>
-      <c r="D33" s="4" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>Loyalty SaaS; IPO attempted — verify state</t>
         </is>
       </c>
-      <c r="E33" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F33" s="6" t="n"/>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="4" t="n">
+      <c r="A34" s="2" t="n">
         <v>33</v>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -3305,25 +3086,25 @@
           <t>Perfios</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>India profitable</t>
         </is>
       </c>
-      <c r="D34" s="4" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>Profitable fintech data SaaS, IPO-bound</t>
         </is>
       </c>
-      <c r="E34" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F34" s="6" t="n"/>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="n">
+      <c r="A35" s="2" t="n">
         <v>34</v>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -3331,25 +3112,25 @@
           <t>IDfy</t>
         </is>
       </c>
-      <c r="C35" s="4" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>India profitable</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>Identity verification; steady</t>
         </is>
       </c>
-      <c r="E35" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F35" s="6" t="n"/>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="4" t="n">
+      <c r="A36" s="2" t="n">
         <v>35</v>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -3357,25 +3138,25 @@
           <t>SuperOps</t>
         </is>
       </c>
-      <c r="C36" s="4" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>Earlier-stage</t>
         </is>
       </c>
-      <c r="D36" s="4" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>Chennai MSP SaaS; outbound US motion; growing</t>
         </is>
       </c>
-      <c r="E36" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F36" s="6" t="n"/>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="n">
+      <c r="A37" s="2" t="n">
         <v>36</v>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -3383,25 +3164,25 @@
           <t>Zluri</t>
         </is>
       </c>
-      <c r="C37" s="4" t="inlineStr">
+      <c r="C37" s="2" t="inlineStr">
         <is>
           <t>Earlier-stage</t>
         </is>
       </c>
-      <c r="D37" s="4" t="inlineStr">
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>SaaS management; outbound US</t>
         </is>
       </c>
-      <c r="E37" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F37" s="6" t="n"/>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="4" t="n">
+      <c r="A38" s="2" t="n">
         <v>37</v>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -3409,25 +3190,25 @@
           <t>Spendflo</t>
         </is>
       </c>
-      <c r="C38" s="4" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr">
         <is>
           <t>Earlier-stage</t>
         </is>
       </c>
-      <c r="D38" s="4" t="inlineStr">
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>SaaS buying; Chennai/US</t>
         </is>
       </c>
-      <c r="E38" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F38" s="6" t="n"/>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="4" t="n">
+      <c r="A39" s="2" t="n">
         <v>38</v>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -3435,25 +3216,25 @@
           <t>Fyle</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr">
+      <c r="C39" s="2" t="inlineStr">
         <is>
           <t>Earlier-stage</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>Expense management; sells US via channel</t>
         </is>
       </c>
-      <c r="E39" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F39" s="6" t="n"/>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="4" t="n">
+      <c r="A40" s="2" t="n">
         <v>39</v>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -3461,25 +3242,25 @@
           <t>Zenskar</t>
         </is>
       </c>
-      <c r="C40" s="4" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>Earlier-stage</t>
         </is>
       </c>
-      <c r="D40" s="4" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>Billing (YC); early but sharp team</t>
         </is>
       </c>
-      <c r="E40" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F40" s="6" t="n"/>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="4" t="n">
+      <c r="A41" s="2" t="n">
         <v>40</v>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -3487,25 +3268,25 @@
           <t>Scrut Automation</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>Earlier-stage</t>
         </is>
       </c>
-      <c r="D41" s="4" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>Sprinto competitor; growing</t>
         </is>
       </c>
-      <c r="E41" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F41" s="6" t="n"/>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="4" t="n">
+      <c r="A42" s="2" t="n">
         <v>41</v>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -3513,25 +3294,25 @@
           <t>Facilio</t>
         </is>
       </c>
-      <c r="C42" s="4" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr">
         <is>
           <t>Earlier-stage</t>
         </is>
       </c>
-      <c r="D42" s="4" t="inlineStr">
+      <c r="D42" s="2" t="inlineStr">
         <is>
           <t>Property ops SaaS; Chennai/NY</t>
         </is>
       </c>
-      <c r="E42" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F42" s="6" t="n"/>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="4" t="n">
+      <c r="A43" s="2" t="n">
         <v>42</v>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -3539,25 +3320,25 @@
           <t>Locus</t>
         </is>
       </c>
-      <c r="C43" s="4" t="inlineStr">
+      <c r="C43" s="2" t="inlineStr">
         <is>
           <t>Earlier-stage</t>
         </is>
       </c>
-      <c r="D43" s="4" t="inlineStr">
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>Logistics SaaS; steady</t>
         </is>
       </c>
-      <c r="E43" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F43" s="6" t="n"/>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="4" t="n">
+      <c r="A44" s="2" t="n">
         <v>43</v>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -3565,25 +3346,25 @@
           <t>Shipsy</t>
         </is>
       </c>
-      <c r="C44" s="4" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr">
         <is>
           <t>Earlier-stage</t>
         </is>
       </c>
-      <c r="D44" s="4" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>Logistics SaaS; Gurgaon</t>
         </is>
       </c>
-      <c r="E44" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F44" s="6" t="n"/>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="4" t="n">
+      <c r="A45" s="2" t="n">
         <v>44</v>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -3591,25 +3372,25 @@
           <t>Exotel</t>
         </is>
       </c>
-      <c r="C45" s="4" t="inlineStr">
+      <c r="C45" s="2" t="inlineStr">
         <is>
           <t>Earlier-stage</t>
         </is>
       </c>
-      <c r="D45" s="4" t="inlineStr">
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>CPaaS; profitable-ish, domestic-heavy</t>
         </is>
       </c>
-      <c r="E45" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F45" s="6" t="n"/>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="4" t="n">
+      <c r="A46" s="2" t="n">
         <v>45</v>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -3617,25 +3398,25 @@
           <t>Gupshup</t>
         </is>
       </c>
-      <c r="C46" s="4" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>Earlier-stage</t>
         </is>
       </c>
-      <c r="D46" s="4" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>Conversational messaging; profitability claimed</t>
         </is>
       </c>
-      <c r="E46" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F46" s="6" t="n"/>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="4" t="n">
+      <c r="A47" s="2" t="n">
         <v>46</v>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -3643,25 +3424,25 @@
           <t>Observe.AI</t>
         </is>
       </c>
-      <c r="C47" s="4" t="inlineStr">
+      <c r="C47" s="2" t="inlineStr">
         <is>
           <t>Earlier-stage</t>
         </is>
       </c>
-      <c r="D47" s="4" t="inlineStr">
+      <c r="D47" s="2" t="inlineStr">
         <is>
           <t>Contact-center AI; US-facing</t>
         </is>
       </c>
-      <c r="E47" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F47" s="6" t="n"/>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="4" t="n">
+      <c r="A48" s="2" t="n">
         <v>47</v>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -3669,25 +3450,25 @@
           <t>Yellow.ai</t>
         </is>
       </c>
-      <c r="C48" s="4" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>Earlier-stage</t>
         </is>
       </c>
-      <c r="D48" s="4" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>Conversational AI; verify momentum</t>
         </is>
       </c>
-      <c r="E48" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F48" s="6" t="n"/>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="4" t="n">
+      <c r="A49" s="2" t="n">
         <v>48</v>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -3695,25 +3476,25 @@
           <t>Uniphore</t>
         </is>
       </c>
-      <c r="C49" s="4" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr">
         <is>
           <t>Earlier-stage</t>
         </is>
       </c>
-      <c r="D49" s="4" t="inlineStr">
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>Big raises; revenue questions persist — diligence hard</t>
         </is>
       </c>
-      <c r="E49" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F49" s="6" t="n"/>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="4" t="n">
+      <c r="A50" s="2" t="n">
         <v>49</v>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -3721,25 +3502,25 @@
           <t>Icertis</t>
         </is>
       </c>
-      <c r="C50" s="4" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr">
         <is>
           <t>Earlier-stage</t>
         </is>
       </c>
-      <c r="D50" s="4" t="inlineStr">
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>Pune CLM leader; growth slowed, still solid enterprise logo</t>
         </is>
       </c>
-      <c r="E50" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F50" s="6" t="n"/>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="4" t="n">
+      <c r="A51" s="2" t="n">
         <v>50</v>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -3747,22 +3528,22 @@
           <t>Hasura</t>
         </is>
       </c>
-      <c r="C51" s="4" t="inlineStr">
+      <c r="C51" s="2" t="inlineStr">
         <is>
           <t>Earlier-stage</t>
         </is>
       </c>
-      <c r="D51" s="4" t="inlineStr">
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t>Pivoted to PromptQL/AI — interesting but unproven motion</t>
         </is>
       </c>
-      <c r="E51" s="6" t="inlineStr">
-        <is>
-          <t>Bench</t>
-        </is>
-      </c>
-      <c r="F51" s="6" t="n"/>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Bench</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -3784,138 +3565,133 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="95" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>B2B SaaS Job-Search Target List — Criteria &amp; Legend</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>Built July 2026. Reference package: Rs29 LPA (comp annotated, not filtered). Target roles: SDR/BDR Manager or Account Executive. Based in Bangalore — Tier 1 is sorted Bangalore-first, then remote-friendly, then relocation-required.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr"/>
+      <c r="A3" s="7" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>HOW TO USE THIS WORKBOOK</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>Yellow cells are yours to edit: Status, Next Step, and My Notes columns on both target sheets.</t>
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Yellow cells are yours to fill: RepVue Score, Glassdoor (Sales), G2, Contact Name/LinkedIn, Status, Last Touch, Next Step, My Notes.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>Status column has a dropdown. Row 2 of Tier 1 (Rippling) shows example values in the yellow columns — replace them with your real progress.</t>
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Fill the three review-score columns during your 15-min diligence pass so the sheet accumulates real numbers over time.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>Everything else is research data as of July 2026 — refresh the 'verify' items before outreach.</t>
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Status has a dropdown. Row 2 (Rippling) shows example values marked '(example)' — replace with your real progress.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr"/>
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Research columns (Location, Why, Role Fit, Comp, Risk, Who to Reach, Angle) are data as of July 2026 — refresh 'verify' items before outreach.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
-        <is>
-          <t>SELECTION SIGNALS (what each column reflects)</t>
-        </is>
-      </c>
+      <c r="A9" s="7" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>Growth signal</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>GTM headcount trend, revenue growth, funding news — a company adding salespeople is one where sales is working</t>
+          <t>SELECTION SIGNALS</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>Funding / profitability</t>
-        </is>
-      </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>Runway = fewer layoff surprises. Source: Tracxn, press releases</t>
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Why It Made the List</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Growth signal + funding/profitability in one place: GTM headcount trend, revenue growth, funding news</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>Reviews check</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>G2 momentum (Grid movement, review growth), Glassdoor FILTERED TO SALES DEPT, RepVue score + quota attainment</t>
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Role Fit</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Outbound-led orgs value BDR leadership; enterprise ACV = higher OTE</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t>Risk flags</t>
-        </is>
-      </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Comp Signal</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Known ranges. Benchmarks: India AE avg ~Rs24L; top 10% &gt;Rs45L; Enterprise AE median OTE ~Rs65L (RepVue, 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Risk Flags</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Layoff history (18-24 mo), culture intensity, category risk</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="8" t="inlineStr">
-        <is>
-          <t>Role fit</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>Outbound-led orgs value BDR leadership; enterprise ACV = higher OTE</t>
-        </is>
-      </c>
-    </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>Comp signal</t>
-        </is>
-      </c>
-      <c r="B15" s="8" t="inlineStr">
-        <is>
-          <t>Known ranges. Benchmarks: India AE avg ~Rs24L; top 10% &gt;Rs45L; Enterprise AE median OTE ~Rs65L (RepVue, 2026)</t>
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>RepVue / Glassdoor / G2</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>You fill these: RepVue score + quota attainment; Glassdoor FILTERED TO SALES DEPT; G2 rating + review momentum</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="inlineStr"/>
+      <c r="A16" s="7" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
@@ -3925,130 +3701,130 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>RepVue score + quota attainment (repvue.com)</t>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>RepVue score + quota attainment (repvue.com) — record in col I</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B19" s="8" t="inlineStr">
-        <is>
-          <t>Glassdoor filtered to sales department, last 12 months</t>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Glassdoor filtered to sales department, last 12 months — record in col J</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>LinkedIn: GTM headcount 6-month trend + average sales-rep tenure</t>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>G2 rating + review count trend — record in col K</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="A21" s="7" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B21" s="8" t="inlineStr">
-        <is>
-          <t>Last funding round / layoffs.fyi check</t>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>LinkedIn: GTM headcount 6-month trend + avg sales-rep tenure; last funding / layoffs.fyi check — note anomalies in Risk or Notes</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="inlineStr"/>
+      <c r="A22" s="7" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="9" t="inlineStr">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>KEY SOURCES</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="inlineStr">
+      <c r="A24" s="7" t="inlineStr">
         <is>
           <t>RepVue rankings &amp; salaries</t>
         </is>
       </c>
-      <c r="B24" s="8" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>repvue.com/rankings/overall ; repvue.com/salaries/account-executive/IN</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="inlineStr">
+      <c r="A25" s="7" t="inlineStr">
         <is>
           <t>Rippling India roles &amp; comp</t>
         </is>
       </c>
-      <c r="B25" s="8" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>in.linkedin.com/jobs/rippling-jobs-bengaluru ; 6figr.com/in/salary/rippling</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="inlineStr">
+      <c r="A26" s="7" t="inlineStr">
         <is>
           <t>Rocketlane Series C (Mar 2026)</t>
         </is>
       </c>
-      <c r="B26" s="8" t="inlineStr">
+      <c r="B26" s="7" t="inlineStr">
         <is>
           <t>rocketlane.com/press/rocketlane-raises-series-c</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="inlineStr">
+      <c r="A27" s="7" t="inlineStr">
         <is>
           <t>MoEngage $280M Series F (Dec 2025)</t>
         </is>
       </c>
-      <c r="B27" s="8" t="inlineStr">
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>startupwired.com/2025/12/17/moengage-raises-180m-more-weeks-after-100m-funding/</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="inlineStr">
+      <c r="A28" s="7" t="inlineStr">
         <is>
           <t>Layoff trackers</t>
         </is>
       </c>
-      <c r="B28" s="8" t="inlineStr">
+      <c r="B28" s="7" t="inlineStr">
         <is>
           <t>techcrunch.com/2025/12/22/tech-layoffs-2025-list/ ; trueup.io/layoffs</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="inlineStr">
+      <c r="A29" s="7" t="inlineStr">
         <is>
           <t>India SaaS market data</t>
         </is>
       </c>
-      <c r="B29" s="8" t="inlineStr">
+      <c r="B29" s="7" t="inlineStr">
         <is>
           <t>tracxn.com — $1.26B raised across 103 rounds by Apr 2026 (+38% YoY)</t>
         </is>

</xml_diff>